<commit_message>
Add PDF export, AI report chat widget, and report generation backend
- Add download dropdown with CSV and PDF plot export options
- Add ReportChat widget for AI-powered report generation
- Add report_generator backend blueprint with OpenAI integration
- Update chart components with forwardRef for PDF capture
- Add jspdf and fpdf2 dependencies
- Update prediction database and GA Excel files

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/Combined_sheet_output_speed/GA/GA_2024.xlsx
+++ b/backend/Combined_sheet_output_speed/GA/GA_2024.xlsx
@@ -4069,10 +4069,10 @@
         <v>196.2035105142857</v>
       </c>
       <c r="D93" t="n">
-        <v>5.691074737075248</v>
+        <v>5.691074737075247</v>
       </c>
       <c r="E93" t="n">
-        <v>34.47565171409406</v>
+        <v>34.47565171409407</v>
       </c>
     </row>
     <row r="94">
@@ -4493,7 +4493,7 @@
         <v>1.170435024901576</v>
       </c>
       <c r="E17" t="n">
-        <v>27.12030829661201</v>
+        <v>27.120308296612</v>
       </c>
     </row>
     <row r="18">
@@ -6070,10 +6070,10 @@
         <v>30.61020132263733</v>
       </c>
       <c r="D2" t="n">
-        <v>1.339637886661133</v>
+        <v>1.339637886661134</v>
       </c>
       <c r="E2" t="n">
-        <v>22.84960856021259</v>
+        <v>22.84960856021258</v>
       </c>
     </row>
     <row r="3">
@@ -6089,10 +6089,10 @@
         <v>30.8829702606593</v>
       </c>
       <c r="D3" t="n">
-        <v>1.351575467616795</v>
+        <v>1.351575467616796</v>
       </c>
       <c r="E3" t="n">
-        <v>22.84960847588821</v>
+        <v>22.8496084758882</v>
       </c>
     </row>
     <row r="4">
@@ -6146,7 +6146,7 @@
         <v>8.891330181098876</v>
       </c>
       <c r="D6" t="n">
-        <v>0.389124004159705</v>
+        <v>0.3891240041597052</v>
       </c>
       <c r="E6" t="n">
         <v>22.84960600233153</v>
@@ -6165,7 +6165,7 @@
         <v>8.553209237802173</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3743263406205204</v>
+        <v>0.3743263406205205</v>
       </c>
       <c r="E7" t="n">
         <v>22.84960557043227</v>
@@ -6184,7 +6184,7 @@
         <v>8.362770709450526</v>
       </c>
       <c r="D8" t="n">
-        <v>0.3659919108581624</v>
+        <v>0.3659919108581625</v>
       </c>
       <c r="E8" t="n">
         <v>22.84960530914974</v>
@@ -6203,7 +6203,7 @@
         <v>8.762165989450523</v>
       </c>
       <c r="D9" t="n">
-        <v>0.3834712095278112</v>
+        <v>0.3834712095278113</v>
       </c>
       <c r="E9" t="n">
         <v>22.84960584196099</v>
@@ -6225,7 +6225,7 @@
         <v>0.1491087224935169</v>
       </c>
       <c r="E10" t="n">
-        <v>22.84958673440881</v>
+        <v>22.84958673440879</v>
       </c>
     </row>
     <row r="11">
@@ -6241,10 +6241,10 @@
         <v>3.464937085714264</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1516411235056714</v>
+        <v>0.1516411235056715</v>
       </c>
       <c r="E11" t="n">
-        <v>22.84958727297134</v>
+        <v>22.84958727297133</v>
       </c>
     </row>
     <row r="12">
@@ -6263,7 +6263,7 @@
         <v>0.1536923880863102</v>
       </c>
       <c r="E12" t="n">
-        <v>22.84958769596347</v>
+        <v>22.84958769596348</v>
       </c>
     </row>
     <row r="13">
@@ -6282,7 +6282,7 @@
         <v>0.1483807001011803</v>
       </c>
       <c r="E13" t="n">
-        <v>22.84958657611714</v>
+        <v>22.84958657611713</v>
       </c>
     </row>
     <row r="14">
@@ -6298,7 +6298,7 @@
         <v>3.875575657582396</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1696124767085144</v>
+        <v>0.1696124767085145</v>
       </c>
       <c r="E14" t="n">
         <v>22.84959062441333</v>
@@ -6320,7 +6320,7 @@
         <v>0.1678531282467341</v>
       </c>
       <c r="E15" t="n">
-        <v>22.84959032867342</v>
+        <v>22.84959032867341</v>
       </c>
     </row>
     <row r="16">
@@ -6336,7 +6336,7 @@
         <v>3.767189516043935</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1648690215882371</v>
+        <v>0.164869021588237</v>
       </c>
       <c r="E16" t="n">
         <v>22.84958981228474</v>
@@ -6374,10 +6374,10 @@
         <v>10.7662046452747</v>
       </c>
       <c r="D18" t="n">
-        <v>0.4711767804384162</v>
+        <v>0.4711767804384164</v>
       </c>
       <c r="E18" t="n">
-        <v>22.84960781653345</v>
+        <v>22.84960781653344</v>
       </c>
     </row>
     <row r="19">
@@ -6393,7 +6393,7 @@
         <v>10.21891783912085</v>
       </c>
       <c r="D19" t="n">
-        <v>0.4472250954914167</v>
+        <v>0.4472250954914168</v>
       </c>
       <c r="E19" t="n">
         <v>22.84960737252942</v>
@@ -6412,10 +6412,10 @@
         <v>10.76738327208788</v>
       </c>
       <c r="D20" t="n">
-        <v>0.4712283623474754</v>
+        <v>0.4712283623474757</v>
       </c>
       <c r="E20" t="n">
-        <v>22.84960781742633</v>
+        <v>22.84960781742631</v>
       </c>
     </row>
     <row r="21">
@@ -6431,10 +6431,10 @@
         <v>11.09893384615382</v>
       </c>
       <c r="D21" t="n">
-        <v>0.4857384782130515</v>
+        <v>0.4857384782130518</v>
       </c>
       <c r="E21" t="n">
-        <v>22.84960805860983</v>
+        <v>22.84960805860982</v>
       </c>
     </row>
     <row r="22">
@@ -6450,10 +6450,10 @@
         <v>54.09432631780217</v>
       </c>
       <c r="D22" t="n">
-        <v>2.367408649358135</v>
+        <v>2.367408649358136</v>
       </c>
       <c r="E22" t="n">
-        <v>22.84959393574427</v>
+        <v>22.84959393574426</v>
       </c>
     </row>
     <row r="23">
@@ -6469,10 +6469,10 @@
         <v>53.07156695999997</v>
       </c>
       <c r="D23" t="n">
-        <v>2.32264804111807</v>
+        <v>2.322648041118071</v>
       </c>
       <c r="E23" t="n">
-        <v>22.84959495389259</v>
+        <v>22.84959495389258</v>
       </c>
     </row>
     <row r="24">
@@ -6491,7 +6491,7 @@
         <v>2.409087392318296</v>
       </c>
       <c r="E24" t="n">
-        <v>22.84959294687103</v>
+        <v>22.84959294687102</v>
       </c>
     </row>
     <row r="25">
@@ -6526,10 +6526,10 @@
         <v>138.4873043960439</v>
       </c>
       <c r="D26" t="n">
-        <v>6.061046644566486</v>
+        <v>6.061046644566487</v>
       </c>
       <c r="E26" t="n">
-        <v>22.84874420496217</v>
+        <v>22.84874420496216</v>
       </c>
     </row>
     <row r="27">
@@ -6545,10 +6545,10 @@
         <v>139.7071534443956</v>
       </c>
       <c r="D27" t="n">
-        <v>6.114447461896395</v>
+        <v>6.114447461896398</v>
       </c>
       <c r="E27" t="n">
-        <v>22.84869635645957</v>
+        <v>22.84869635645956</v>
       </c>
     </row>
     <row r="28">
@@ -6564,10 +6564,10 @@
         <v>146.5498341824176</v>
       </c>
       <c r="D28" t="n">
-        <v>6.414015943449161</v>
+        <v>6.414015943449163</v>
       </c>
       <c r="E28" t="n">
-        <v>22.84837385415196</v>
+        <v>22.84837385415195</v>
       </c>
     </row>
     <row r="29">
@@ -6583,7 +6583,7 @@
         <v>161.3237490065934</v>
       </c>
       <c r="D29" t="n">
-        <v>7.060977310917817</v>
+        <v>7.060977310917818</v>
       </c>
       <c r="E29" t="n">
         <v>22.8472266519185</v>
@@ -6602,10 +6602,10 @@
         <v>223.4656607881318</v>
       </c>
       <c r="D30" t="n">
-        <v>9.797117149620167</v>
+        <v>9.797117149620169</v>
       </c>
       <c r="E30" t="n">
-        <v>22.80932823149875</v>
+        <v>22.80932823149874</v>
       </c>
     </row>
     <row r="31">
@@ -6621,7 +6621,7 @@
         <v>227.0606436593406</v>
       </c>
       <c r="D31" t="n">
-        <v>9.957931729957526</v>
+        <v>9.957931729957529</v>
       </c>
       <c r="E31" t="n">
         <v>22.80198838642862</v>
@@ -6643,7 +6643,7 @@
         <v>10.03690710232164</v>
       </c>
       <c r="E32" t="n">
-        <v>22.79791092562209</v>
+        <v>22.79791092562208</v>
       </c>
     </row>
     <row r="33">
@@ -6659,10 +6659,10 @@
         <v>229.7645977292308</v>
       </c>
       <c r="D33" t="n">
-        <v>10.07934938515903</v>
+        <v>10.07934938515904</v>
       </c>
       <c r="E33" t="n">
-        <v>22.79557826098768</v>
+        <v>22.79557826098767</v>
       </c>
     </row>
     <row r="34">
@@ -6678,10 +6678,10 @@
         <v>263.2762170738461</v>
       </c>
       <c r="D34" t="n">
-        <v>11.66041180274352</v>
+        <v>11.66041180274353</v>
       </c>
       <c r="E34" t="n">
-        <v>22.57863800418276</v>
+        <v>22.57863800418275</v>
       </c>
     </row>
     <row r="35">
@@ -6700,7 +6700,7 @@
         <v>12.01094184081939</v>
       </c>
       <c r="E35" t="n">
-        <v>22.46953243511504</v>
+        <v>22.46953243511503</v>
       </c>
     </row>
     <row r="36">
@@ -6716,10 +6716,10 @@
         <v>266.8434463727472</v>
       </c>
       <c r="D36" t="n">
-        <v>11.846654189603</v>
+        <v>11.84665418960301</v>
       </c>
       <c r="E36" t="n">
-        <v>22.52479409814608</v>
+        <v>22.52479409814607</v>
       </c>
     </row>
     <row r="37">
@@ -6754,10 +6754,10 @@
         <v>275.7965023806593</v>
       </c>
       <c r="D38" t="n">
-        <v>12.35190426487596</v>
+        <v>12.35190426487597</v>
       </c>
       <c r="E38" t="n">
-        <v>22.32825777033569</v>
+        <v>22.32825777033568</v>
       </c>
     </row>
     <row r="39">
@@ -6773,10 +6773,10 @@
         <v>271.9631481771428</v>
       </c>
       <c r="D39" t="n">
-        <v>12.12739822235165</v>
+        <v>12.12739822235166</v>
       </c>
       <c r="E39" t="n">
-        <v>22.42551478815097</v>
+        <v>22.42551478815096</v>
       </c>
     </row>
     <row r="40">
@@ -6814,7 +6814,7 @@
         <v>11.98618959695453</v>
       </c>
       <c r="E41" t="n">
-        <v>22.4783564237574</v>
+        <v>22.47835642375739</v>
       </c>
     </row>
     <row r="42">
@@ -6871,7 +6871,7 @@
         <v>13.20000053719058</v>
       </c>
       <c r="E44" t="n">
-        <v>21.79273481071968</v>
+        <v>21.79273481071967</v>
       </c>
     </row>
     <row r="45">
@@ -6890,7 +6890,7 @@
         <v>13.27723237766576</v>
       </c>
       <c r="E45" t="n">
-        <v>21.73017792834329</v>
+        <v>21.73017792834328</v>
       </c>
     </row>
     <row r="46">
@@ -6906,10 +6906,10 @@
         <v>313.1479132272528</v>
       </c>
       <c r="D46" t="n">
-        <v>15.64101465240685</v>
+        <v>15.64101465240686</v>
       </c>
       <c r="E46" t="n">
-        <v>20.02094622288877</v>
+        <v>20.02094622288876</v>
       </c>
     </row>
     <row r="47">
@@ -6928,7 +6928,7 @@
         <v>15.74819828987271</v>
       </c>
       <c r="E47" t="n">
-        <v>19.95269772843421</v>
+        <v>19.9526977284342</v>
       </c>
     </row>
     <row r="48">
@@ -6944,10 +6944,10 @@
         <v>314.7991741450549</v>
       </c>
       <c r="D48" t="n">
-        <v>15.80640289460823</v>
+        <v>15.80640289460824</v>
       </c>
       <c r="E48" t="n">
-        <v>19.91592750381157</v>
+        <v>19.91592750381156</v>
       </c>
     </row>
     <row r="49">
@@ -6963,10 +6963,10 @@
         <v>314.3879723986813</v>
       </c>
       <c r="D49" t="n">
-        <v>15.80640289460823</v>
+        <v>15.80640289460824</v>
       </c>
       <c r="E49" t="n">
-        <v>19.88991261926666</v>
+        <v>19.88991261926665</v>
       </c>
     </row>
     <row r="50">
@@ -6982,10 +6982,10 @@
         <v>359.3116791296703</v>
       </c>
       <c r="D50" t="n">
-        <v>20.64637778088954</v>
+        <v>20.64637778088955</v>
       </c>
       <c r="E50" t="n">
-        <v>17.40313399972039</v>
+        <v>17.40313399972038</v>
       </c>
     </row>
     <row r="51">
@@ -7001,10 +7001,10 @@
         <v>358.0589865520879</v>
       </c>
       <c r="D51" t="n">
-        <v>20.64637778088954</v>
+        <v>20.64637778088955</v>
       </c>
       <c r="E51" t="n">
-        <v>17.34246027811766</v>
+        <v>17.34246027811765</v>
       </c>
     </row>
     <row r="52">
@@ -7020,10 +7020,10 @@
         <v>357.6618475345055</v>
       </c>
       <c r="D52" t="n">
-        <v>20.64637778088954</v>
+        <v>20.64637778088955</v>
       </c>
       <c r="E52" t="n">
-        <v>17.32322499036903</v>
+        <v>17.32322499036902</v>
       </c>
     </row>
     <row r="53">
@@ -7039,10 +7039,10 @@
         <v>355.9815260993406</v>
       </c>
       <c r="D53" t="n">
-        <v>20.64637778088954</v>
+        <v>20.64637778088955</v>
       </c>
       <c r="E53" t="n">
-        <v>17.24183921640919</v>
+        <v>17.24183921640918</v>
       </c>
     </row>
     <row r="54">
@@ -7058,10 +7058,10 @@
         <v>349.8871248712088</v>
       </c>
       <c r="D54" t="n">
-        <v>20.64637778088954</v>
+        <v>20.64637778088955</v>
       </c>
       <c r="E54" t="n">
-        <v>16.94665905004738</v>
+        <v>16.94665905004737</v>
       </c>
     </row>
     <row r="55">
@@ -7077,10 +7077,10 @@
         <v>352.418698829011</v>
       </c>
       <c r="D55" t="n">
-        <v>20.94622832107846</v>
+        <v>20.94622832107848</v>
       </c>
       <c r="E55" t="n">
-        <v>16.82492396372704</v>
+        <v>16.82492396372703</v>
       </c>
     </row>
     <row r="56">
@@ -7096,10 +7096,10 @@
         <v>349.4623142624176</v>
       </c>
       <c r="D56" t="n">
-        <v>20.94622832107846</v>
+        <v>20.94622832107848</v>
       </c>
       <c r="E56" t="n">
-        <v>16.68378234523249</v>
+        <v>16.68378234523248</v>
       </c>
     </row>
     <row r="57">
@@ -7115,10 +7115,10 @@
         <v>349.6339589208791</v>
       </c>
       <c r="D57" t="n">
-        <v>20.9668096027182</v>
+        <v>20.96680960271821</v>
       </c>
       <c r="E57" t="n">
-        <v>16.67559183041141</v>
+        <v>16.6755918304114</v>
       </c>
     </row>
     <row r="58">
@@ -7134,10 +7134,10 @@
         <v>355.2095671213186</v>
       </c>
       <c r="D58" t="n">
-        <v>21.64085647713941</v>
+        <v>21.64085647713943</v>
       </c>
       <c r="E58" t="n">
-        <v>16.41384052874934</v>
+        <v>16.41384052874933</v>
       </c>
     </row>
     <row r="59">
@@ -7153,10 +7153,10 @@
         <v>355.5885918804395</v>
       </c>
       <c r="D59" t="n">
-        <v>21.68706467281215</v>
+        <v>21.68706467281216</v>
       </c>
       <c r="E59" t="n">
-        <v>16.39634488323452</v>
+        <v>16.39634488323451</v>
       </c>
     </row>
     <row r="60">
@@ -7172,10 +7172,10 @@
         <v>348.4196655771428</v>
       </c>
       <c r="D60" t="n">
-        <v>21.68706467281215</v>
+        <v>21.68706467281216</v>
       </c>
       <c r="E60" t="n">
-        <v>16.0657825682577</v>
+        <v>16.06578256825769</v>
       </c>
     </row>
     <row r="61">
@@ -7191,10 +7191,10 @@
         <v>349.3192596210989</v>
       </c>
       <c r="D61" t="n">
-        <v>21.79919806974794</v>
+        <v>21.79919806974796</v>
       </c>
       <c r="E61" t="n">
-        <v>16.02440871923038</v>
+        <v>16.02440871923037</v>
       </c>
     </row>
     <row r="62">
@@ -7210,10 +7210,10 @@
         <v>356.8486793907691</v>
       </c>
       <c r="D62" t="n">
-        <v>22.74906979780212</v>
+        <v>22.74906979780213</v>
       </c>
       <c r="E62" t="n">
-        <v>15.68629761843035</v>
+        <v>15.68629761843034</v>
       </c>
     </row>
     <row r="63">
@@ -7229,10 +7229,10 @@
         <v>358.3253799745054</v>
       </c>
       <c r="D63" t="n">
-        <v>22.9377384102348</v>
+        <v>22.93773841023481</v>
       </c>
       <c r="E63" t="n">
-        <v>15.6216525607695</v>
+        <v>15.62165256076949</v>
       </c>
     </row>
     <row r="64">
@@ -7248,10 +7248,10 @@
         <v>354.358451233846</v>
       </c>
       <c r="D64" t="n">
-        <v>22.9377384102348</v>
+        <v>22.93773841023481</v>
       </c>
       <c r="E64" t="n">
-        <v>15.4487092361177</v>
+        <v>15.44870923611769</v>
       </c>
     </row>
     <row r="65">
@@ -7267,10 +7267,10 @@
         <v>352.5632267538461</v>
       </c>
       <c r="D65" t="n">
-        <v>22.9377384102348</v>
+        <v>22.93773841023481</v>
       </c>
       <c r="E65" t="n">
-        <v>15.37044413221369</v>
+        <v>15.37044413221368</v>
       </c>
     </row>
     <row r="66">
@@ -7286,10 +7286,10 @@
         <v>373.7397727279121</v>
       </c>
       <c r="D66" t="n">
-        <v>25.77598114035739</v>
+        <v>25.77598114035741</v>
       </c>
       <c r="E66" t="n">
-        <v>14.4995362423954</v>
+        <v>14.49953624239538</v>
       </c>
     </row>
     <row r="67">
@@ -7305,10 +7305,10 @@
         <v>373.2558834501098</v>
       </c>
       <c r="D67" t="n">
-        <v>25.77598114035738</v>
+        <v>25.7759811403574</v>
       </c>
       <c r="E67" t="n">
-        <v>14.48076336716836</v>
+        <v>14.48076336716835</v>
       </c>
     </row>
     <row r="68">
@@ -7324,10 +7324,10 @@
         <v>373.7905071468131</v>
       </c>
       <c r="D68" t="n">
-        <v>25.84987318051506</v>
+        <v>25.84987318051508</v>
       </c>
       <c r="E68" t="n">
-        <v>14.46005187478314</v>
+        <v>14.46005187478313</v>
       </c>
     </row>
     <row r="69">
@@ -7343,10 +7343,10 @@
         <v>375.2396454474725</v>
       </c>
       <c r="D69" t="n">
-        <v>26.05069505525815</v>
+        <v>26.05069505525817</v>
       </c>
       <c r="E69" t="n">
-        <v>14.40420858835139</v>
+        <v>14.40420858835138</v>
       </c>
     </row>
     <row r="70">
@@ -7362,10 +7362,10 @@
         <v>370.5674071740658</v>
       </c>
       <c r="D70" t="n">
-        <v>25.40600146870595</v>
+        <v>25.40600146870596</v>
       </c>
       <c r="E70" t="n">
-        <v>14.58582168589242</v>
+        <v>14.58582168589241</v>
       </c>
     </row>
     <row r="71">
@@ -7381,10 +7381,10 @@
         <v>370.6651749810989</v>
       </c>
       <c r="D71" t="n">
-        <v>25.40600146870595</v>
+        <v>25.40600146870596</v>
       </c>
       <c r="E71" t="n">
-        <v>14.58966990290341</v>
+        <v>14.5896699029034</v>
       </c>
     </row>
     <row r="72">
@@ -7400,10 +7400,10 @@
         <v>374.37187908</v>
       </c>
       <c r="D72" t="n">
-        <v>25.40600146870595</v>
+        <v>25.40600146870596</v>
       </c>
       <c r="E72" t="n">
-        <v>14.73556866243339</v>
+        <v>14.73556866243338</v>
       </c>
     </row>
     <row r="73">
@@ -7419,10 +7419,10 @@
         <v>374.6524932527472</v>
       </c>
       <c r="D73" t="n">
-        <v>25.40600146870595</v>
+        <v>25.40600146870596</v>
       </c>
       <c r="E73" t="n">
-        <v>14.74661385477083</v>
+        <v>14.74661385477082</v>
       </c>
     </row>
     <row r="74">
@@ -7441,7 +7441,7 @@
         <v>20.97430976998552</v>
       </c>
       <c r="E74" t="n">
-        <v>16.22992932939863</v>
+        <v>16.22992932939862</v>
       </c>
     </row>
     <row r="75">
@@ -7457,10 +7457,10 @@
         <v>337.3097902246154</v>
       </c>
       <c r="D75" t="n">
-        <v>20.59382214415265</v>
+        <v>20.59382214415266</v>
       </c>
       <c r="E75" t="n">
-        <v>16.3791737086741</v>
+        <v>16.37917370867409</v>
       </c>
     </row>
     <row r="76">
@@ -7476,10 +7476,10 @@
         <v>337.4643875670329</v>
       </c>
       <c r="D76" t="n">
-        <v>20.59382214415265</v>
+        <v>20.59382214415266</v>
       </c>
       <c r="E76" t="n">
-        <v>16.3866806853458</v>
+        <v>16.38668068534579</v>
       </c>
     </row>
     <row r="77">
@@ -7495,10 +7495,10 @@
         <v>337.4051128562637</v>
       </c>
       <c r="D77" t="n">
-        <v>20.58658828072593</v>
+        <v>20.58658828072594</v>
       </c>
       <c r="E77" t="n">
-        <v>16.38955946732355</v>
+        <v>16.38955946732354</v>
       </c>
     </row>
     <row r="78">
@@ -7517,7 +7517,7 @@
         <v>12.59805847935922</v>
       </c>
       <c r="E78" t="n">
-        <v>22.20122132749056</v>
+        <v>22.20122132749055</v>
       </c>
     </row>
     <row r="79">
@@ -7536,7 +7536,7 @@
         <v>12.51603357187028</v>
       </c>
       <c r="E79" t="n">
-        <v>22.24603320795041</v>
+        <v>22.2460332079504</v>
       </c>
     </row>
     <row r="80">
@@ -7555,7 +7555,7 @@
         <v>12.42511964104743</v>
       </c>
       <c r="E80" t="n">
-        <v>22.29278342953694</v>
+        <v>22.29278342953693</v>
       </c>
     </row>
     <row r="81">
@@ -7574,7 +7574,7 @@
         <v>12.29512509585927</v>
       </c>
       <c r="E81" t="n">
-        <v>22.35446698484215</v>
+        <v>22.35446698484214</v>
       </c>
     </row>
     <row r="82">
@@ -7590,10 +7590,10 @@
         <v>213.7335229516484</v>
       </c>
       <c r="D82" t="n">
-        <v>9.364444672973406</v>
+        <v>9.364444672973407</v>
       </c>
       <c r="E82" t="n">
-        <v>22.8239399575398</v>
+        <v>22.82393995753979</v>
       </c>
     </row>
     <row r="83">
@@ -7609,10 +7609,10 @@
         <v>212.4219156672527</v>
       </c>
       <c r="D83" t="n">
-        <v>9.306364248388739</v>
+        <v>9.306364248388743</v>
       </c>
       <c r="E83" t="n">
-        <v>22.82544611382801</v>
+        <v>22.825446113828</v>
       </c>
     </row>
     <row r="84">
@@ -7628,10 +7628,10 @@
         <v>213.8133749182417</v>
       </c>
       <c r="D84" t="n">
-        <v>9.367982155594127</v>
+        <v>9.367982155594131</v>
       </c>
       <c r="E84" t="n">
-        <v>22.8238452387062</v>
+        <v>22.82384523870619</v>
       </c>
     </row>
     <row r="85">
@@ -7647,10 +7647,10 @@
         <v>213.4275219652748</v>
       </c>
       <c r="D85" t="n">
-        <v>9.350890282891452</v>
+        <v>9.350890282891458</v>
       </c>
       <c r="E85" t="n">
-        <v>22.82429966649972</v>
+        <v>22.8242996664997</v>
       </c>
     </row>
     <row r="86">
@@ -7666,10 +7666,10 @@
         <v>157.1992609107692</v>
       </c>
       <c r="D86" t="n">
-        <v>6.880332110156038</v>
+        <v>6.880332110156041</v>
       </c>
       <c r="E86" t="n">
-        <v>22.84762688689516</v>
+        <v>22.84762688689515</v>
       </c>
     </row>
     <row r="87">
@@ -7685,7 +7685,7 @@
         <v>156.2733735085714</v>
       </c>
       <c r="D87" t="n">
-        <v>6.839783698075112</v>
+        <v>6.839783698075113</v>
       </c>
       <c r="E87" t="n">
         <v>22.84770694613496</v>
@@ -7704,10 +7704,10 @@
         <v>156.2389913485714</v>
       </c>
       <c r="D88" t="n">
-        <v>6.838277986665286</v>
+        <v>6.838277986665289</v>
       </c>
       <c r="E88" t="n">
-        <v>22.8477098552061</v>
+        <v>22.84770985520609</v>
       </c>
     </row>
     <row r="89">
@@ -7723,7 +7723,7 @@
         <v>156.7579186351648</v>
       </c>
       <c r="D89" t="n">
-        <v>6.861003758597583</v>
+        <v>6.861003758597586</v>
       </c>
       <c r="E89" t="n">
         <v>22.84766546567331</v>
@@ -7742,10 +7742,10 @@
         <v>99.50524790769229</v>
       </c>
       <c r="D90" t="n">
-        <v>4.354819408693424</v>
+        <v>4.354819408693426</v>
       </c>
       <c r="E90" t="n">
-        <v>22.84945449380801</v>
+        <v>22.849454493808</v>
       </c>
     </row>
     <row r="91">
@@ -7761,7 +7761,7 @@
         <v>100.3838488496703</v>
       </c>
       <c r="D91" t="n">
-        <v>4.393272326514579</v>
+        <v>4.39327232651458</v>
       </c>
       <c r="E91" t="n">
         <v>22.84944829024752</v>
@@ -7780,10 +7780,10 @@
         <v>99.95495938417579</v>
       </c>
       <c r="D92" t="n">
-        <v>4.374501508275402</v>
+        <v>4.374501508275404</v>
       </c>
       <c r="E92" t="n">
-        <v>22.84945134779069</v>
+        <v>22.84945134779068</v>
       </c>
     </row>
     <row r="93">
@@ -7799,10 +7799,10 @@
         <v>101.8805136131868</v>
       </c>
       <c r="D93" t="n">
-        <v>4.458775630484695</v>
+        <v>4.458775630484696</v>
       </c>
       <c r="E93" t="n">
-        <v>22.84943716760016</v>
+        <v>22.84943716760015</v>
       </c>
     </row>
     <row r="94">
@@ -7818,10 +7818,10 @@
         <v>62.4277858140659</v>
       </c>
       <c r="D94" t="n">
-        <v>2.732119168847426</v>
+        <v>2.732119168847428</v>
       </c>
       <c r="E94" t="n">
-        <v>22.84958376848611</v>
+        <v>22.8495837684861</v>
       </c>
     </row>
     <row r="95">
@@ -7837,7 +7837,7 @@
         <v>62.82371174901096</v>
       </c>
       <c r="D95" t="n">
-        <v>2.749446728368237</v>
+        <v>2.749446728368238</v>
       </c>
       <c r="E95" t="n">
         <v>22.8495831909775</v>
@@ -7875,10 +7875,10 @@
         <v>64.24512974505491</v>
       </c>
       <c r="D97" t="n">
-        <v>2.811654605017022</v>
+        <v>2.811654605017023</v>
       </c>
       <c r="E97" t="n">
-        <v>22.84958103688059</v>
+        <v>22.84958103688058</v>
       </c>
     </row>
   </sheetData>
@@ -8201,7 +8201,7 @@
         <v>29.73550933450547</v>
       </c>
       <c r="D16" t="n">
-        <v>1.36757739048477</v>
+        <v>1.367577390484771</v>
       </c>
       <c r="E16" t="n">
         <v>21.74320045168706</v>
@@ -9898,7 +9898,7 @@
         <v>1.69278012320381</v>
       </c>
       <c r="E7" t="n">
-        <v>50.80135384759658</v>
+        <v>50.80135384759659</v>
       </c>
     </row>
     <row r="8">
@@ -12520,7 +12520,7 @@
         <v>886.1867469217582</v>
       </c>
       <c r="D47" t="n">
-        <v>24.5146043949178</v>
+        <v>24.51460439491779</v>
       </c>
       <c r="E47" t="n">
         <v>36.14933908970102</v>
@@ -12558,10 +12558,10 @@
         <v>882.9076835617583</v>
       </c>
       <c r="D49" t="n">
-        <v>23.02039947266763</v>
+        <v>23.02039947266762</v>
       </c>
       <c r="E49" t="n">
-        <v>38.35327378267455</v>
+        <v>38.35327378267456</v>
       </c>
     </row>
     <row r="50">
@@ -12710,10 +12710,10 @@
         <v>956.9201780650548</v>
       </c>
       <c r="D57" t="n">
-        <v>26.48066679529901</v>
+        <v>26.48066679529898</v>
       </c>
       <c r="E57" t="n">
-        <v>36.13655900216729</v>
+        <v>36.13655900216732</v>
       </c>
     </row>
     <row r="58">
@@ -13549,7 +13549,7 @@
         <v>159.970558294945</v>
       </c>
       <c r="D3" t="n">
-        <v>3.097782632988745</v>
+        <v>3.097782632988746</v>
       </c>
       <c r="E3" t="n">
         <v>51.64034318980126</v>
@@ -14312,7 +14312,7 @@
         <v>20.6195859462152</v>
       </c>
       <c r="E43" t="n">
-        <v>29.67954999234207</v>
+        <v>29.67954999234206</v>
       </c>
     </row>
     <row r="44">
@@ -14404,10 +14404,10 @@
         <v>635.4690135942856</v>
       </c>
       <c r="D48" t="n">
-        <v>20.62770722371686</v>
+        <v>20.62770722371687</v>
       </c>
       <c r="E48" t="n">
-        <v>30.80657519046277</v>
+        <v>30.80657519046276</v>
       </c>
     </row>
     <row r="49">
@@ -15398,7 +15398,7 @@
         <v>1.820265680860277</v>
       </c>
       <c r="E2" t="n">
-        <v>44.72506916959536</v>
+        <v>44.72506916959535</v>
       </c>
     </row>
     <row r="3">
@@ -15547,10 +15547,10 @@
         <v>39.26279422681316</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8782236739649278</v>
+        <v>0.878223673964928</v>
       </c>
       <c r="E10" t="n">
-        <v>44.70705515094226</v>
+        <v>44.70705515094225</v>
       </c>
     </row>
     <row r="11">
@@ -15585,10 +15585,10 @@
         <v>39.06507957890107</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8738130900206208</v>
+        <v>0.8738130900206209</v>
       </c>
       <c r="E12" t="n">
-        <v>44.70644812379635</v>
+        <v>44.70644812379634</v>
       </c>
     </row>
     <row r="13">
@@ -15642,10 +15642,10 @@
         <v>40.99139777670326</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9167877245148059</v>
+        <v>0.9167877245148061</v>
       </c>
       <c r="E15" t="n">
-        <v>44.71198368018862</v>
+        <v>44.71198368018861</v>
       </c>
     </row>
     <row r="16">
@@ -15661,7 +15661,7 @@
         <v>40.48648212923074</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9055228781791316</v>
+        <v>0.9055228781791317</v>
       </c>
       <c r="E16" t="n">
         <v>44.71061207270972</v>
@@ -15680,10 +15680,10 @@
         <v>42.27254017186809</v>
       </c>
       <c r="D17" t="n">
-        <v>0.9453723377361275</v>
+        <v>0.9453723377361274</v>
       </c>
       <c r="E17" t="n">
-        <v>44.71522857660259</v>
+        <v>44.7152285766026</v>
       </c>
     </row>
     <row r="18">
@@ -15927,7 +15927,7 @@
         <v>326.1173515885714</v>
       </c>
       <c r="D30" t="n">
-        <v>8.018276470510139</v>
+        <v>8.018276470510138</v>
       </c>
       <c r="E30" t="n">
         <v>40.67175193920735</v>
@@ -15946,10 +15946,10 @@
         <v>324.2464074646153</v>
       </c>
       <c r="D31" t="n">
-        <v>7.946580022795576</v>
+        <v>7.946580022795573</v>
       </c>
       <c r="E31" t="n">
-        <v>40.80326461628542</v>
+        <v>40.80326461628543</v>
       </c>
     </row>
     <row r="32">
@@ -15965,10 +15965,10 @@
         <v>319.2360458716483</v>
       </c>
       <c r="D32" t="n">
-        <v>7.761683856325791</v>
+        <v>7.76168385632579</v>
       </c>
       <c r="E32" t="n">
-        <v>41.12974088882403</v>
+        <v>41.12974088882404</v>
       </c>
     </row>
     <row r="33">
@@ -15984,10 +15984,10 @@
         <v>326.00526204</v>
       </c>
       <c r="D33" t="n">
-        <v>8.013936827213081</v>
+        <v>8.01393682721308</v>
       </c>
       <c r="E33" t="n">
-        <v>40.67978935558583</v>
+        <v>40.67978935558584</v>
       </c>
     </row>
     <row r="34">
@@ -16003,10 +16003,10 @@
         <v>355.4561805243956</v>
       </c>
       <c r="D34" t="n">
-        <v>9.490166662544075</v>
+        <v>9.49016666254407</v>
       </c>
       <c r="E34" t="n">
-        <v>37.45520949882947</v>
+        <v>37.45520949882949</v>
       </c>
     </row>
     <row r="35">
@@ -16022,10 +16022,10 @@
         <v>359.0433217252747</v>
       </c>
       <c r="D35" t="n">
-        <v>9.759111073797213</v>
+        <v>9.759111073797207</v>
       </c>
       <c r="E35" t="n">
-        <v>36.79057641728153</v>
+        <v>36.79057641728155</v>
       </c>
     </row>
     <row r="36">
@@ -16041,7 +16041,7 @@
         <v>361.4715793002197</v>
       </c>
       <c r="D36" t="n">
-        <v>9.965435595615281</v>
+        <v>9.965435595615279</v>
       </c>
       <c r="E36" t="n">
         <v>36.27253177565711</v>
@@ -16063,7 +16063,7 @@
         <v>10.08348261519677</v>
       </c>
       <c r="E37" t="n">
-        <v>35.97391999097246</v>
+        <v>35.97391999097248</v>
       </c>
     </row>
     <row r="38">
@@ -16079,10 +16079,10 @@
         <v>368.2786968751648</v>
       </c>
       <c r="D38" t="n">
-        <v>10.72016529063768</v>
+        <v>10.72016529063767</v>
       </c>
       <c r="E38" t="n">
-        <v>34.35382635347948</v>
+        <v>34.35382635347952</v>
       </c>
     </row>
     <row r="39">
@@ -16098,10 +16098,10 @@
         <v>367.3143270698901</v>
       </c>
       <c r="D39" t="n">
-        <v>10.59024266086115</v>
+        <v>10.59024266086114</v>
       </c>
       <c r="E39" t="n">
-        <v>34.68422196097459</v>
+        <v>34.6842219609746</v>
       </c>
     </row>
     <row r="40">
@@ -16117,10 +16117,10 @@
         <v>366.5890842487912</v>
       </c>
       <c r="D40" t="n">
-        <v>10.49895456276678</v>
+        <v>10.49895456276677</v>
       </c>
       <c r="E40" t="n">
-        <v>34.91672261815984</v>
+        <v>34.91672261815987</v>
       </c>
     </row>
     <row r="41">
@@ -16139,7 +16139,7 @@
         <v>10.29912897066958</v>
       </c>
       <c r="E41" t="n">
-        <v>35.42584617606715</v>
+        <v>35.42584617606716</v>
       </c>
     </row>
     <row r="42">
@@ -16177,7 +16177,7 @@
         <v>11.659698346108</v>
       </c>
       <c r="E43" t="n">
-        <v>33.200155688851</v>
+        <v>33.20015568885101</v>
       </c>
     </row>
     <row r="44">
@@ -16196,7 +16196,7 @@
         <v>11.659698346108</v>
       </c>
       <c r="E44" t="n">
-        <v>33.17710941030693</v>
+        <v>33.17710941030694</v>
       </c>
     </row>
     <row r="45">
@@ -16212,10 +16212,10 @@
         <v>386.840043418022</v>
       </c>
       <c r="D45" t="n">
-        <v>11.65999709002232</v>
+        <v>11.65999709002231</v>
       </c>
       <c r="E45" t="n">
-        <v>33.176684387773</v>
+        <v>33.17668438777301</v>
       </c>
     </row>
     <row r="46">
@@ -16234,7 +16234,7 @@
         <v>12.98655619110549</v>
       </c>
       <c r="E46" t="n">
-        <v>31.43657348568708</v>
+        <v>31.43657348568709</v>
       </c>
     </row>
     <row r="47">
@@ -16272,7 +16272,7 @@
         <v>13.08933214593559</v>
       </c>
       <c r="E48" t="n">
-        <v>31.20644637664552</v>
+        <v>31.20644637664553</v>
       </c>
     </row>
     <row r="49">
@@ -16288,10 +16288,10 @@
         <v>410.8768778531868</v>
       </c>
       <c r="D49" t="n">
-        <v>13.2439423933353</v>
+        <v>13.24394239333529</v>
       </c>
       <c r="E49" t="n">
-        <v>31.02375906285661</v>
+        <v>31.02375906285662</v>
       </c>
     </row>
     <row r="50">
@@ -16842,7 +16842,7 @@
         <v>13.64106764145922</v>
       </c>
       <c r="E78" t="n">
-        <v>30.83453724442678</v>
+        <v>30.83453724442677</v>
       </c>
     </row>
     <row r="79">
@@ -16855,13 +16855,13 @@
         <v>375.7576008421977</v>
       </c>
       <c r="C79" t="n">
-        <v>401.1420841510562</v>
+        <v>401.1420841510563</v>
       </c>
       <c r="D79" t="n">
-        <v>12.40718393359743</v>
+        <v>12.40718393359744</v>
       </c>
       <c r="E79" t="n">
-        <v>32.33143687543819</v>
+        <v>32.33143687543817</v>
       </c>
     </row>
     <row r="80">
@@ -16874,13 +16874,13 @@
         <v>375.2319023920878</v>
       </c>
       <c r="C80" t="n">
-        <v>381.6681600577931</v>
+        <v>381.6681600577932</v>
       </c>
       <c r="D80" t="n">
-        <v>11.23178108011159</v>
+        <v>11.2317810801116</v>
       </c>
       <c r="E80" t="n">
-        <v>33.98108967184403</v>
+        <v>33.98108967184401</v>
       </c>
     </row>
     <row r="81">
@@ -16896,10 +16896,10 @@
         <v>370.9064916923076</v>
       </c>
       <c r="D81" t="n">
-        <v>11.1406893323284</v>
+        <v>11.14068933232838</v>
       </c>
       <c r="E81" t="n">
-        <v>33.29295707187523</v>
+        <v>33.29295707187526</v>
       </c>
     </row>
     <row r="82">
@@ -16915,10 +16915,10 @@
         <v>309.8524061221977</v>
       </c>
       <c r="D82" t="n">
-        <v>7.438362165073412</v>
+        <v>7.438362165073411</v>
       </c>
       <c r="E82" t="n">
-        <v>41.6559988940979</v>
+        <v>41.65599889409791</v>
       </c>
     </row>
     <row r="83">
@@ -16953,10 +16953,10 @@
         <v>306.6639413815385</v>
       </c>
       <c r="D84" t="n">
-        <v>7.334079404880689</v>
+        <v>7.334079404880686</v>
       </c>
       <c r="E84" t="n">
-        <v>41.81355620140403</v>
+        <v>41.81355620140405</v>
       </c>
     </row>
     <row r="85">
@@ -16972,10 +16972,10 @@
         <v>309.0563090571429</v>
       </c>
       <c r="D85" t="n">
-        <v>7.412088082434233</v>
+        <v>7.412088082434232</v>
       </c>
       <c r="E85" t="n">
-        <v>41.69625422956989</v>
+        <v>41.6962542295699</v>
       </c>
     </row>
     <row r="86">
@@ -17010,10 +17010,10 @@
         <v>242.9158202663736</v>
       </c>
       <c r="D87" t="n">
-        <v>5.562932831851892</v>
+        <v>5.562932831851891</v>
       </c>
       <c r="E87" t="n">
-        <v>43.66686199687715</v>
+        <v>43.66686199687716</v>
       </c>
     </row>
     <row r="88">
@@ -17032,7 +17032,7 @@
         <v>5.497454971511043</v>
       </c>
       <c r="E88" t="n">
-        <v>43.71020664956544</v>
+        <v>43.71020664956545</v>
       </c>
     </row>
     <row r="89">
@@ -17048,10 +17048,10 @@
         <v>237.8689248065933</v>
       </c>
       <c r="D89" t="n">
-        <v>5.437144224148089</v>
+        <v>5.437144224148088</v>
       </c>
       <c r="E89" t="n">
-        <v>43.74887165033101</v>
+        <v>43.74887165033102</v>
       </c>
     </row>
     <row r="90">
@@ -17086,10 +17086,10 @@
         <v>177.8669074312087</v>
       </c>
       <c r="D91" t="n">
-        <v>4.007682068430383</v>
+        <v>4.007682068430382</v>
       </c>
       <c r="E91" t="n">
-        <v>44.38149144422292</v>
+        <v>44.38149144422294</v>
       </c>
     </row>
     <row r="92">
@@ -17143,10 +17143,10 @@
         <v>126.6238148215384</v>
       </c>
       <c r="D94" t="n">
-        <v>2.837327583076174</v>
+        <v>2.837327583076175</v>
       </c>
       <c r="E94" t="n">
-        <v>44.62784472854396</v>
+        <v>44.62784472854395</v>
       </c>
     </row>
     <row r="95">
@@ -17162,10 +17162,10 @@
         <v>126.2645593885714</v>
       </c>
       <c r="D95" t="n">
-        <v>2.829204416427379</v>
+        <v>2.82920441642738</v>
       </c>
       <c r="E95" t="n">
-        <v>44.62899840514667</v>
+        <v>44.62899840514666</v>
       </c>
     </row>
     <row r="96">
@@ -17526,10 +17526,10 @@
         <v>18.621741661978</v>
       </c>
       <c r="D16" t="n">
-        <v>0.6757281054966087</v>
+        <v>0.6757281054966088</v>
       </c>
       <c r="E16" t="n">
-        <v>27.55803926239303</v>
+        <v>27.55803926239302</v>
       </c>
     </row>
     <row r="17">
@@ -23390,7 +23390,7 @@
         <v>14.73481664071972</v>
       </c>
       <c r="E30" t="n">
-        <v>44.91717488346737</v>
+        <v>44.91717488346736</v>
       </c>
     </row>
     <row r="31">
@@ -23580,7 +23580,7 @@
         <v>18.6983032232002</v>
       </c>
       <c r="E40" t="n">
-        <v>38.14473108690226</v>
+        <v>38.14473108690227</v>
       </c>
     </row>
     <row r="41">
@@ -23672,10 +23672,10 @@
         <v>753.9345874786814</v>
       </c>
       <c r="D45" t="n">
-        <v>24.65702128837261</v>
+        <v>24.65702128837262</v>
       </c>
       <c r="E45" t="n">
-        <v>30.57687214774035</v>
+        <v>30.57687214774034</v>
       </c>
     </row>
     <row r="46">
@@ -26645,7 +26645,7 @@
         <v>1.950953788585696</v>
       </c>
       <c r="E5" t="n">
-        <v>17.63168434334251</v>
+        <v>17.63168434334252</v>
       </c>
     </row>
     <row r="6">
@@ -26661,10 +26661,10 @@
         <v>18.82210584395602</v>
       </c>
       <c r="D6" t="n">
-        <v>1.067555721595734</v>
+        <v>1.067555721595735</v>
       </c>
       <c r="E6" t="n">
-        <v>17.63102896008237</v>
+        <v>17.63102896008236</v>
       </c>
     </row>
     <row r="7">
@@ -26737,7 +26737,7 @@
         <v>14.24225314021976</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8078363696900435</v>
+        <v>0.8078363696900437</v>
       </c>
       <c r="E10" t="n">
         <v>17.63012124062244</v>
@@ -26794,7 +26794,7 @@
         <v>13.94441224351646</v>
       </c>
       <c r="D13" t="n">
-        <v>0.7909463333715731</v>
+        <v>0.7909463333715732</v>
       </c>
       <c r="E13" t="n">
         <v>17.63003588887694</v>
@@ -26832,7 +26832,7 @@
         <v>14.93218111780217</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8469610931524456</v>
+        <v>0.8469610931524457</v>
       </c>
       <c r="E15" t="n">
         <v>17.63030349153772</v>
@@ -26851,7 +26851,7 @@
         <v>15.2575617230769</v>
       </c>
       <c r="D16" t="n">
-        <v>0.8654129685162603</v>
+        <v>0.8654129685162604</v>
       </c>
       <c r="E16" t="n">
         <v>17.6303825781994</v>
@@ -26870,7 +26870,7 @@
         <v>14.92485509670327</v>
       </c>
       <c r="D17" t="n">
-        <v>0.8465456452435166</v>
+        <v>0.8465456452435167</v>
       </c>
       <c r="E17" t="n">
         <v>17.63030166248153</v>
@@ -26930,7 +26930,7 @@
         <v>1.32257239082003</v>
       </c>
       <c r="E20" t="n">
-        <v>17.63146792285391</v>
+        <v>17.63146792285392</v>
       </c>
     </row>
     <row r="21">
@@ -26965,7 +26965,7 @@
         <v>54.4823416707692</v>
       </c>
       <c r="D22" t="n">
-        <v>3.090218557000249</v>
+        <v>3.090218557000248</v>
       </c>
       <c r="E22" t="n">
         <v>17.63057876516558</v>
@@ -27041,10 +27041,10 @@
         <v>137.6859652931868</v>
       </c>
       <c r="D26" t="n">
-        <v>7.823253140948955</v>
+        <v>7.823253140948957</v>
       </c>
       <c r="E26" t="n">
-        <v>17.59957946042963</v>
+        <v>17.59957946042962</v>
       </c>
     </row>
     <row r="27">
@@ -27079,7 +27079,7 @@
         <v>145.4823309665934</v>
       </c>
       <c r="D28" t="n">
-        <v>8.270022597790607</v>
+        <v>8.270022597790609</v>
       </c>
       <c r="E28" t="n">
         <v>17.59152762236224</v>
@@ -27098,7 +27098,7 @@
         <v>147.3403351463736</v>
       </c>
       <c r="D29" t="n">
-        <v>8.376680926737711</v>
+        <v>8.376680926737713</v>
       </c>
       <c r="E29" t="n">
         <v>17.58934552181339</v>
@@ -27155,7 +27155,7 @@
         <v>234.9429207718681</v>
       </c>
       <c r="D32" t="n">
-        <v>13.72902850525163</v>
+        <v>13.72902850525162</v>
       </c>
       <c r="E32" t="n">
         <v>17.11285839941244</v>
@@ -27326,7 +27326,7 @@
         <v>270.1830462395604</v>
       </c>
       <c r="D41" t="n">
-        <v>17.07102601785775</v>
+        <v>17.07102601785776</v>
       </c>
       <c r="E41" t="n">
         <v>15.82699516460966</v>
@@ -27345,7 +27345,7 @@
         <v>274.9312061393406</v>
       </c>
       <c r="D42" t="n">
-        <v>17.9054568036542</v>
+        <v>17.90545680365421</v>
       </c>
       <c r="E42" t="n">
         <v>15.3546044177567</v>
@@ -27364,10 +27364,10 @@
         <v>275.4136197573625</v>
       </c>
       <c r="D43" t="n">
-        <v>18.00772225973985</v>
+        <v>18.00772225973986</v>
       </c>
       <c r="E43" t="n">
-        <v>15.29419522274114</v>
+        <v>15.29419522274113</v>
       </c>
     </row>
     <row r="44">
@@ -27386,7 +27386,7 @@
         <v>18.17743058766879</v>
       </c>
       <c r="E44" t="n">
-        <v>15.19303261609004</v>
+        <v>15.19303261609005</v>
       </c>
     </row>
     <row r="45">
@@ -27402,7 +27402,7 @@
         <v>279.3751460624176</v>
       </c>
       <c r="D45" t="n">
-        <v>19.08060323837802</v>
+        <v>19.08060323837801</v>
       </c>
       <c r="E45" t="n">
         <v>14.64184033241113</v>
@@ -27440,10 +27440,10 @@
         <v>300.1338842769231</v>
       </c>
       <c r="D47" t="n">
-        <v>22.02148609564698</v>
+        <v>22.02148609564697</v>
       </c>
       <c r="E47" t="n">
-        <v>13.62913851378318</v>
+        <v>13.62913851378319</v>
       </c>
     </row>
     <row r="48">
@@ -27459,7 +27459,7 @@
         <v>299.9727902294506</v>
       </c>
       <c r="D48" t="n">
-        <v>22.02148609564698</v>
+        <v>22.02148609564697</v>
       </c>
       <c r="E48" t="n">
         <v>13.62182320151167</v>
@@ -27478,7 +27478,7 @@
         <v>298.456295545055</v>
       </c>
       <c r="D49" t="n">
-        <v>22.02148609564698</v>
+        <v>22.02148609564697</v>
       </c>
       <c r="E49" t="n">
         <v>13.55295888064754</v>
@@ -27497,10 +27497,10 @@
         <v>334.8351848136264</v>
       </c>
       <c r="D50" t="n">
-        <v>27.7170694952267</v>
+        <v>27.71706949522669</v>
       </c>
       <c r="E50" t="n">
-        <v>12.08046849510155</v>
+        <v>12.08046849510156</v>
       </c>
     </row>
     <row r="51">
@@ -27516,10 +27516,10 @@
         <v>334.5702706153846</v>
       </c>
       <c r="D51" t="n">
-        <v>27.7170694952267</v>
+        <v>27.71706949522669</v>
       </c>
       <c r="E51" t="n">
-        <v>12.07091069541109</v>
+        <v>12.0709106954111</v>
       </c>
     </row>
     <row r="52">
@@ -27535,7 +27535,7 @@
         <v>332.1410708518681</v>
       </c>
       <c r="D52" t="n">
-        <v>27.7170694952267</v>
+        <v>27.71706949522669</v>
       </c>
       <c r="E52" t="n">
         <v>11.98326796088843</v>
@@ -27554,10 +27554,10 @@
         <v>336.8704927239561</v>
       </c>
       <c r="D53" t="n">
-        <v>28.51202684252052</v>
+        <v>28.51202684252051</v>
       </c>
       <c r="E53" t="n">
-        <v>11.81503141058968</v>
+        <v>11.81503141058969</v>
       </c>
     </row>
     <row r="54">
@@ -27573,10 +27573,10 @@
         <v>334.7220841648352</v>
       </c>
       <c r="D54" t="n">
-        <v>28.51202684252052</v>
+        <v>28.5120268425205</v>
       </c>
       <c r="E54" t="n">
-        <v>11.73968045181754</v>
+        <v>11.73968045181755</v>
       </c>
     </row>
     <row r="55">
@@ -27592,10 +27592,10 @@
         <v>331.9499550883516</v>
       </c>
       <c r="D55" t="n">
-        <v>28.51202684252052</v>
+        <v>28.51202684252051</v>
       </c>
       <c r="E55" t="n">
-        <v>11.64245379403573</v>
+        <v>11.64245379403574</v>
       </c>
     </row>
     <row r="56">
@@ -27611,7 +27611,7 @@
         <v>329.9367262325274</v>
       </c>
       <c r="D56" t="n">
-        <v>28.51202684252052</v>
+        <v>28.51202684252051</v>
       </c>
       <c r="E56" t="n">
         <v>11.57184398200996</v>
@@ -27630,7 +27630,7 @@
         <v>327.5751335485714</v>
       </c>
       <c r="D57" t="n">
-        <v>28.51202684252052</v>
+        <v>28.51202684252051</v>
       </c>
       <c r="E57" t="n">
         <v>11.48901603375501</v>
@@ -27649,7 +27649,7 @@
         <v>333.6696250747253</v>
       </c>
       <c r="D58" t="n">
-        <v>29.58282091361333</v>
+        <v>29.58282091361332</v>
       </c>
       <c r="E58" t="n">
         <v>11.27916861103595</v>
@@ -27668,7 +27668,7 @@
         <v>334.0981961208792</v>
       </c>
       <c r="D59" t="n">
-        <v>29.6588630924264</v>
+        <v>29.65886309242638</v>
       </c>
       <c r="E59" t="n">
         <v>11.26470003518758</v>
@@ -27687,10 +27687,10 @@
         <v>332.6221133657143</v>
       </c>
       <c r="D60" t="n">
-        <v>29.6588630924264</v>
+        <v>29.65886309242638</v>
       </c>
       <c r="E60" t="n">
-        <v>11.21493134545173</v>
+        <v>11.21493134545174</v>
       </c>
     </row>
     <row r="61">
@@ -27706,7 +27706,7 @@
         <v>331.4517690197802</v>
       </c>
       <c r="D61" t="n">
-        <v>29.6588630924264</v>
+        <v>29.65886309242638</v>
       </c>
       <c r="E61" t="n">
         <v>11.17547115635794</v>
@@ -27725,7 +27725,7 @@
         <v>338.4070822826374</v>
       </c>
       <c r="D62" t="n">
-        <v>30.91666952731508</v>
+        <v>30.91666952731506</v>
       </c>
       <c r="E62" t="n">
         <v>10.94578062438623</v>
@@ -27744,7 +27744,7 @@
         <v>337.7041371323077</v>
       </c>
       <c r="D63" t="n">
-        <v>30.91666952731508</v>
+        <v>30.91666952731506</v>
       </c>
       <c r="E63" t="n">
         <v>10.92304385612894</v>
@@ -27763,10 +27763,10 @@
         <v>339.2915739824176</v>
       </c>
       <c r="D64" t="n">
-        <v>31.20801100358216</v>
+        <v>31.20801100358215</v>
       </c>
       <c r="E64" t="n">
-        <v>10.87193842451134</v>
+        <v>10.87193842451135</v>
       </c>
     </row>
     <row r="65">
@@ -27782,7 +27782,7 @@
         <v>334.6419351652748</v>
       </c>
       <c r="D65" t="n">
-        <v>31.20801100358216</v>
+        <v>31.20801100358215</v>
       </c>
       <c r="E65" t="n">
         <v>10.72294979410458</v>
@@ -27801,10 +27801,10 @@
         <v>356.4361516892307</v>
       </c>
       <c r="D66" t="n">
-        <v>35.40534711718645</v>
+        <v>35.40534711718643</v>
       </c>
       <c r="E66" t="n">
-        <v>10.06729719410686</v>
+        <v>10.06729719410687</v>
       </c>
     </row>
     <row r="67">
@@ -27820,7 +27820,7 @@
         <v>349.9236171534065</v>
       </c>
       <c r="D67" t="n">
-        <v>34.12336679346627</v>
+        <v>34.12336679346624</v>
       </c>
       <c r="E67" t="n">
         <v>10.25466271459497</v>
@@ -27839,10 +27839,10 @@
         <v>344.5782724734066</v>
       </c>
       <c r="D68" t="n">
-        <v>33.08880958551386</v>
+        <v>33.08880958551384</v>
       </c>
       <c r="E68" t="n">
-        <v>10.41374037899089</v>
+        <v>10.4137403789909</v>
       </c>
     </row>
     <row r="69">
@@ -27858,10 +27858,10 @@
         <v>347.7716739019779</v>
       </c>
       <c r="D69" t="n">
-        <v>33.08880958551386</v>
+        <v>33.08880958551384</v>
       </c>
       <c r="E69" t="n">
-        <v>10.5102503915472</v>
+        <v>10.51025039154721</v>
       </c>
     </row>
     <row r="70">
@@ -27877,7 +27877,7 @@
         <v>351.1282640545055</v>
       </c>
       <c r="D70" t="n">
-        <v>33.08880958551386</v>
+        <v>33.08880958551384</v>
       </c>
       <c r="E70" t="n">
         <v>10.61169224438428</v>
@@ -27896,7 +27896,7 @@
         <v>351.6439501173626</v>
       </c>
       <c r="D71" t="n">
-        <v>33.08880958551385</v>
+        <v>33.08880958551383</v>
       </c>
       <c r="E71" t="n">
         <v>10.62727715267554</v>
@@ -27915,10 +27915,10 @@
         <v>345.3280371481318</v>
       </c>
       <c r="D72" t="n">
-        <v>31.91086108567557</v>
+        <v>31.91086108567555</v>
       </c>
       <c r="E72" t="n">
-        <v>10.82164584092485</v>
+        <v>10.82164584092486</v>
       </c>
     </row>
     <row r="73">
@@ -27934,7 +27934,7 @@
         <v>346.9452782861538</v>
       </c>
       <c r="D73" t="n">
-        <v>31.91086108567557</v>
+        <v>31.91086108567555</v>
       </c>
       <c r="E73" t="n">
         <v>10.87232580012997</v>
@@ -27953,10 +27953,10 @@
         <v>312.0884405947253</v>
       </c>
       <c r="D74" t="n">
-        <v>25.82093277484976</v>
+        <v>25.82093277484974</v>
       </c>
       <c r="E74" t="n">
-        <v>12.08664471249107</v>
+        <v>12.08664471249108</v>
       </c>
     </row>
     <row r="75">
@@ -27972,10 +27972,10 @@
         <v>312.3979251837362</v>
       </c>
       <c r="D75" t="n">
-        <v>25.82093277484976</v>
+        <v>25.82093277484975</v>
       </c>
       <c r="E75" t="n">
-        <v>12.09863051454205</v>
+        <v>12.09863051454206</v>
       </c>
     </row>
     <row r="76">
@@ -27991,10 +27991,10 @@
         <v>312.8709050347253</v>
       </c>
       <c r="D76" t="n">
-        <v>25.82093277484976</v>
+        <v>25.82093277484975</v>
       </c>
       <c r="E76" t="n">
-        <v>12.11694820488706</v>
+        <v>12.11694820488707</v>
       </c>
     </row>
     <row r="77">
@@ -28010,10 +28010,10 @@
         <v>310.1984566575824</v>
       </c>
       <c r="D77" t="n">
-        <v>25.381707532585</v>
+        <v>25.38170753258499</v>
       </c>
       <c r="E77" t="n">
-        <v>12.22133917741153</v>
+        <v>12.22133917741154</v>
       </c>
     </row>
     <row r="78">
@@ -28029,7 +28029,7 @@
         <v>254.8038257538461</v>
       </c>
       <c r="D78" t="n">
-        <v>15.31134777954465</v>
+        <v>15.31134777954466</v>
       </c>
       <c r="E78" t="n">
         <v>16.64150206908981</v>
@@ -28067,7 +28067,7 @@
         <v>249.6178962909889</v>
       </c>
       <c r="D80" t="n">
-        <v>14.85611458731971</v>
+        <v>14.8561145873197</v>
       </c>
       <c r="E80" t="n">
         <v>16.80236745777714</v>
@@ -28181,7 +28181,7 @@
         <v>136.3232243775824</v>
       </c>
       <c r="D86" t="n">
-        <v>7.745276202434011</v>
+        <v>7.74527620243401</v>
       </c>
       <c r="E86" t="n">
         <v>17.6008215607265</v>
@@ -28200,10 +28200,10 @@
         <v>137.369090523956</v>
       </c>
       <c r="D87" t="n">
-        <v>7.805118571946696</v>
+        <v>7.805118571946695</v>
       </c>
       <c r="E87" t="n">
-        <v>17.59987234757593</v>
+        <v>17.59987234757594</v>
       </c>
     </row>
     <row r="88">
@@ -28276,7 +28276,7 @@
         <v>92.91088673010984</v>
       </c>
       <c r="D91" t="n">
-        <v>5.271876022452656</v>
+        <v>5.271876022452657</v>
       </c>
       <c r="E91" t="n">
         <v>17.62387551118558</v>
@@ -28333,7 +28333,7 @@
         <v>59.16521491252744</v>
       </c>
       <c r="D94" t="n">
-        <v>3.355917954427953</v>
+        <v>3.355917954427954</v>
       </c>
       <c r="E94" t="n">
         <v>17.63011364281481</v>
@@ -28526,10 +28526,10 @@
         <v>76.0533070285714</v>
       </c>
       <c r="D6" t="n">
-        <v>1.579328664018362</v>
+        <v>1.579328664018361</v>
       </c>
       <c r="E6" t="n">
-        <v>48.15546552233486</v>
+        <v>48.15546552233487</v>
       </c>
     </row>
     <row r="7">
@@ -28716,7 +28716,7 @@
         <v>56.24774166461535</v>
       </c>
       <c r="D16" t="n">
-        <v>1.168664324538962</v>
+        <v>1.168664324538963</v>
       </c>
       <c r="E16" t="n">
         <v>48.12993815551361</v>
@@ -28757,7 +28757,7 @@
         <v>1.547122884465914</v>
       </c>
       <c r="E18" t="n">
-        <v>48.1558973327538</v>
+        <v>48.15589733275382</v>
       </c>
     </row>
     <row r="19">
@@ -30144,7 +30144,7 @@
         <v>5.356825851183538</v>
       </c>
       <c r="E91" t="n">
-        <v>46.30984062081256</v>
+        <v>46.30984062081255</v>
       </c>
     </row>
     <row r="92">
@@ -30429,10 +30429,10 @@
         <v>111.8985373635164</v>
       </c>
       <c r="D8" t="n">
-        <v>2.413964869530941</v>
+        <v>2.413964869530942</v>
       </c>
       <c r="E8" t="n">
-        <v>46.35466687021815</v>
+        <v>46.35466687021813</v>
       </c>
     </row>
     <row r="9">
@@ -34083,10 +34083,10 @@
         <v>47.96235398373623</v>
       </c>
       <c r="D4" t="n">
-        <v>1.813300766623508</v>
+        <v>1.813300766623509</v>
       </c>
       <c r="E4" t="n">
-        <v>26.45030260095542</v>
+        <v>26.45030260095541</v>
       </c>
     </row>
     <row r="5">
@@ -34102,10 +34102,10 @@
         <v>49.0857742496703</v>
       </c>
       <c r="D5" t="n">
-        <v>1.855778014887631</v>
+        <v>1.85577801488763</v>
       </c>
       <c r="E5" t="n">
-        <v>26.45024019892944</v>
+        <v>26.45024019892945</v>
       </c>
     </row>
     <row r="6">
@@ -34121,10 +34121,10 @@
         <v>26.035809272967</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9844417893733159</v>
+        <v>0.9844417893733156</v>
       </c>
       <c r="E6" t="n">
-        <v>26.44728165140276</v>
+        <v>26.44728165140277</v>
       </c>
     </row>
     <row r="7">
@@ -34143,7 +34143,7 @@
         <v>1.003047826500447</v>
       </c>
       <c r="E7" t="n">
-        <v>26.44749601637519</v>
+        <v>26.4474960163752</v>
       </c>
     </row>
     <row r="8">
@@ -34159,10 +34159,10 @@
         <v>26.05054804879119</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9849988328903777</v>
+        <v>0.984998832890378</v>
       </c>
       <c r="E8" t="n">
-        <v>26.44728823926475</v>
+        <v>26.44728823926474</v>
       </c>
     </row>
     <row r="9">
@@ -34181,7 +34181,7 @@
         <v>1.007988826776212</v>
       </c>
       <c r="E9" t="n">
-        <v>26.44755101758414</v>
+        <v>26.44755101758413</v>
       </c>
     </row>
     <row r="10">
@@ -34197,7 +34197,7 @@
         <v>19.80198908703294</v>
       </c>
       <c r="D10" t="n">
-        <v>0.7488484242097345</v>
+        <v>0.7488484242097346</v>
       </c>
       <c r="E10" t="n">
         <v>26.44325399753646</v>
@@ -34216,10 +34216,10 @@
         <v>19.18857086109887</v>
       </c>
       <c r="D11" t="n">
-        <v>0.7256666980073254</v>
+        <v>0.7256666980073259</v>
       </c>
       <c r="E11" t="n">
-        <v>26.44267804184831</v>
+        <v>26.44267804184829</v>
       </c>
     </row>
     <row r="12">
@@ -34254,10 +34254,10 @@
         <v>19.17943293890107</v>
       </c>
       <c r="D13" t="n">
-        <v>0.7253213675734077</v>
+        <v>0.725321367573408</v>
       </c>
       <c r="E13" t="n">
-        <v>26.44266913446469</v>
+        <v>26.44266913446468</v>
       </c>
     </row>
     <row r="14">
@@ -34273,7 +34273,7 @@
         <v>20.41177162945052</v>
       </c>
       <c r="D14" t="n">
-        <v>0.7718929327837257</v>
+        <v>0.7718929327837258</v>
       </c>
       <c r="E14" t="n">
         <v>26.4437861295585</v>
@@ -34292,10 +34292,10 @@
         <v>20.44435495780218</v>
       </c>
       <c r="D15" t="n">
-        <v>0.7731243059776214</v>
+        <v>0.7731243059776216</v>
       </c>
       <c r="E15" t="n">
-        <v>26.44381349768863</v>
+        <v>26.44381349768862</v>
       </c>
     </row>
     <row r="16">
@@ -34311,7 +34311,7 @@
         <v>20.99885491252744</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7940797762753408</v>
+        <v>0.7940797762753407</v>
       </c>
       <c r="E16" t="n">
         <v>26.44426358649167</v>
@@ -34330,7 +34330,7 @@
         <v>20.75522966109886</v>
       </c>
       <c r="D17" t="n">
-        <v>0.7848727565909073</v>
+        <v>0.7848727565909072</v>
       </c>
       <c r="E17" t="n">
         <v>26.44406941992629</v>
@@ -34482,10 +34482,10 @@
         <v>79.5457469907692</v>
       </c>
       <c r="D25" t="n">
-        <v>3.008059327670314</v>
+        <v>3.008059327670313</v>
       </c>
       <c r="E25" t="n">
-        <v>26.44420815076673</v>
+        <v>26.44420815076674</v>
       </c>
     </row>
     <row r="26">
@@ -34501,7 +34501,7 @@
         <v>173.6340593327472</v>
       </c>
       <c r="D26" t="n">
-        <v>6.589133893161904</v>
+        <v>6.589133893161903</v>
       </c>
       <c r="E26" t="n">
         <v>26.35157551024146</v>
@@ -34520,7 +34520,7 @@
         <v>175.4643669705494</v>
       </c>
       <c r="D27" t="n">
-        <v>6.65959490236021</v>
+        <v>6.659594902360209</v>
       </c>
       <c r="E27" t="n">
         <v>26.34760365204249</v>
@@ -34580,7 +34580,7 @@
         <v>10.8481217581227</v>
       </c>
       <c r="E30" t="n">
-        <v>25.58656248355387</v>
+        <v>25.58656248355386</v>
       </c>
     </row>
     <row r="31">
@@ -34653,10 +34653,10 @@
         <v>321.3750883872528</v>
       </c>
       <c r="D34" t="n">
-        <v>13.4111062691302</v>
+        <v>13.41110626913021</v>
       </c>
       <c r="E34" t="n">
-        <v>23.96335409905718</v>
+        <v>23.96335409905717</v>
       </c>
     </row>
     <row r="35">
@@ -34713,7 +34713,7 @@
         <v>13.56812816116157</v>
       </c>
       <c r="E37" t="n">
-        <v>23.82441830312901</v>
+        <v>23.82441830312902</v>
       </c>
     </row>
     <row r="38">
@@ -34767,10 +34767,10 @@
         <v>326.567124847912</v>
       </c>
       <c r="D40" t="n">
-        <v>13.86782067215197</v>
+        <v>13.86782067215198</v>
       </c>
       <c r="E40" t="n">
-        <v>23.54855406399167</v>
+        <v>23.54855406399166</v>
       </c>
     </row>
     <row r="41">
@@ -34805,7 +34805,7 @@
         <v>340.4169772404396</v>
       </c>
       <c r="D42" t="n">
-        <v>15.78672787313547</v>
+        <v>15.78672787313546</v>
       </c>
       <c r="E42" t="n">
         <v>21.56349181262146</v>
@@ -34824,10 +34824,10 @@
         <v>338.6988577661538</v>
       </c>
       <c r="D43" t="n">
-        <v>15.43539806662219</v>
+        <v>15.4353980666222</v>
       </c>
       <c r="E43" t="n">
-        <v>21.94299468690496</v>
+        <v>21.94299468690495</v>
       </c>
     </row>
     <row r="44">
@@ -34862,7 +34862,7 @@
         <v>337.1675648993407</v>
       </c>
       <c r="D45" t="n">
-        <v>15.16636669864806</v>
+        <v>15.16636669864807</v>
       </c>
       <c r="E45" t="n">
         <v>22.23126814739327</v>
@@ -34884,7 +34884,7 @@
         <v>17.3685352317065</v>
       </c>
       <c r="E46" t="n">
-        <v>20.77415732399204</v>
+        <v>20.77415732399203</v>
       </c>
     </row>
     <row r="47">
@@ -34903,7 +34903,7 @@
         <v>17.3685352317065</v>
       </c>
       <c r="E47" t="n">
-        <v>20.71593607324493</v>
+        <v>20.71593607324492</v>
       </c>
     </row>
     <row r="48">
@@ -34919,10 +34919,10 @@
         <v>362.996870912967</v>
       </c>
       <c r="D48" t="n">
-        <v>17.67801281765725</v>
+        <v>17.67801281765726</v>
       </c>
       <c r="E48" t="n">
-        <v>20.53380516561208</v>
+        <v>20.53380516561207</v>
       </c>
     </row>
     <row r="49">
@@ -34938,10 +34938,10 @@
         <v>361.9058664487912</v>
       </c>
       <c r="D49" t="n">
-        <v>17.67801281765725</v>
+        <v>17.67801281765726</v>
       </c>
       <c r="E49" t="n">
-        <v>20.47208983168687</v>
+        <v>20.47208983168686</v>
       </c>
     </row>
     <row r="50">
@@ -35014,7 +35014,7 @@
         <v>408.0451497059341</v>
       </c>
       <c r="D53" t="n">
-        <v>22.85322676346225</v>
+        <v>22.85322676346226</v>
       </c>
       <c r="E53" t="n">
         <v>17.85503438658023</v>
@@ -35033,7 +35033,7 @@
         <v>411.5172417217582</v>
       </c>
       <c r="D54" t="n">
-        <v>23.24380166892377</v>
+        <v>23.24380166892378</v>
       </c>
       <c r="E54" t="n">
         <v>17.70438620941873</v>
@@ -35052,7 +35052,7 @@
         <v>406.9943967731868</v>
       </c>
       <c r="D55" t="n">
-        <v>23.24380166892377</v>
+        <v>23.24380166892378</v>
       </c>
       <c r="E55" t="n">
         <v>17.50980336909884</v>
@@ -35074,7 +35074,7 @@
         <v>23.49272339666867</v>
       </c>
       <c r="E56" t="n">
-        <v>17.41679206665082</v>
+        <v>17.41679206665081</v>
       </c>
     </row>
     <row r="57">
@@ -35109,7 +35109,7 @@
         <v>419.6166915178022</v>
       </c>
       <c r="D58" t="n">
-        <v>24.805052361948</v>
+        <v>24.80505236194801</v>
       </c>
       <c r="E58" t="n">
         <v>16.91658156551654</v>
@@ -35147,7 +35147,7 @@
         <v>421.9856090347253</v>
       </c>
       <c r="D60" t="n">
-        <v>25.42728259270169</v>
+        <v>25.4272825927017</v>
       </c>
       <c r="E60" t="n">
         <v>16.59578083093497</v>
@@ -35166,10 +35166,10 @@
         <v>418.8414437907692</v>
       </c>
       <c r="D61" t="n">
-        <v>25.42728259270169</v>
+        <v>25.4272825927017</v>
       </c>
       <c r="E61" t="n">
-        <v>16.47212761583056</v>
+        <v>16.47212761583055</v>
       </c>
     </row>
     <row r="62">
@@ -35185,10 +35185,10 @@
         <v>429.0346540206593</v>
       </c>
       <c r="D62" t="n">
-        <v>26.67997379553694</v>
+        <v>26.67997379553695</v>
       </c>
       <c r="E62" t="n">
-        <v>16.08077494035728</v>
+        <v>16.08077494035727</v>
       </c>
     </row>
     <row r="63">
@@ -35204,7 +35204,7 @@
         <v>432.2321402465934</v>
       </c>
       <c r="D63" t="n">
-        <v>27.0791338190925</v>
+        <v>27.07913381909251</v>
       </c>
       <c r="E63" t="n">
         <v>15.96181558591222</v>
@@ -35223,10 +35223,10 @@
         <v>435.0898017481318</v>
       </c>
       <c r="D64" t="n">
-        <v>27.43837967857641</v>
+        <v>27.43837967857642</v>
       </c>
       <c r="E64" t="n">
-        <v>15.85697868623945</v>
+        <v>15.85697868623944</v>
       </c>
     </row>
     <row r="65">
@@ -35242,10 +35242,10 @@
         <v>428.9552856237361</v>
       </c>
       <c r="D65" t="n">
-        <v>27.43837967857641</v>
+        <v>27.43837967857642</v>
       </c>
       <c r="E65" t="n">
-        <v>15.63340440101351</v>
+        <v>15.6334044010135</v>
       </c>
     </row>
     <row r="66">
@@ -35261,7 +35261,7 @@
         <v>455.0936698852747</v>
       </c>
       <c r="D66" t="n">
-        <v>30.88417492678299</v>
+        <v>30.884174926783</v>
       </c>
       <c r="E66" t="n">
         <v>14.73549709403485</v>
@@ -35280,10 +35280,10 @@
         <v>450.9030872017581</v>
       </c>
       <c r="D67" t="n">
-        <v>30.31801976484889</v>
+        <v>30.3180197648489</v>
       </c>
       <c r="E67" t="n">
-        <v>14.87244518933064</v>
+        <v>14.87244518933063</v>
       </c>
     </row>
     <row r="68">
@@ -35299,7 +35299,7 @@
         <v>449.4377677331868</v>
       </c>
       <c r="D68" t="n">
-        <v>30.12128836075368</v>
+        <v>30.1212883607537</v>
       </c>
       <c r="E68" t="n">
         <v>14.92093440195534</v>
@@ -35318,7 +35318,7 @@
         <v>441.6806175402197</v>
       </c>
       <c r="D69" t="n">
-        <v>29.09049403691128</v>
+        <v>29.09049403691129</v>
       </c>
       <c r="E69" t="n">
         <v>15.18298785093839</v>
@@ -35337,7 +35337,7 @@
         <v>453.2321048742857</v>
       </c>
       <c r="D70" t="n">
-        <v>29.09049403691128</v>
+        <v>29.09049403691129</v>
       </c>
       <c r="E70" t="n">
         <v>15.58007589349308</v>
@@ -35356,7 +35356,7 @@
         <v>445.9307434523077</v>
       </c>
       <c r="D71" t="n">
-        <v>28.16077447984162</v>
+        <v>28.16077447984163</v>
       </c>
       <c r="E71" t="n">
         <v>15.83517327520658</v>
@@ -35375,10 +35375,10 @@
         <v>450.2238132026373</v>
       </c>
       <c r="D72" t="n">
-        <v>28.16077447984163</v>
+        <v>28.16077447984164</v>
       </c>
       <c r="E72" t="n">
-        <v>15.98762184345895</v>
+        <v>15.98762184345894</v>
       </c>
     </row>
     <row r="73">
@@ -35394,10 +35394,10 @@
         <v>445.5410777841757</v>
       </c>
       <c r="D73" t="n">
-        <v>27.57802576094459</v>
+        <v>27.57802576094461</v>
       </c>
       <c r="E73" t="n">
-        <v>16.15565529042117</v>
+        <v>16.15565529042116</v>
       </c>
     </row>
     <row r="74">
@@ -35413,7 +35413,7 @@
         <v>405.0836300334066</v>
       </c>
       <c r="D74" t="n">
-        <v>22.79696628790177</v>
+        <v>22.79696628790179</v>
       </c>
       <c r="E74" t="n">
         <v>17.76919020353959</v>
@@ -35451,7 +35451,7 @@
         <v>399.7657383283516</v>
       </c>
       <c r="D76" t="n">
-        <v>22.20234320079684</v>
+        <v>22.20234320079685</v>
       </c>
       <c r="E76" t="n">
         <v>18.00556521052264</v>
@@ -35470,10 +35470,10 @@
         <v>394.6167538259339</v>
       </c>
       <c r="D77" t="n">
-        <v>21.63409388778032</v>
+        <v>21.63409388778033</v>
       </c>
       <c r="E77" t="n">
-        <v>18.24050297058325</v>
+        <v>18.24050297058324</v>
       </c>
     </row>
     <row r="78">
@@ -35508,10 +35508,10 @@
         <v>324.0348582092308</v>
       </c>
       <c r="D79" t="n">
-        <v>13.63606214978826</v>
+        <v>13.63606214978827</v>
       </c>
       <c r="E79" t="n">
-        <v>23.76308164701804</v>
+        <v>23.76308164701803</v>
       </c>
     </row>
     <row r="80">
@@ -35584,7 +35584,7 @@
         <v>252.507511410989</v>
       </c>
       <c r="D83" t="n">
-        <v>9.733209220323916</v>
+        <v>9.733209220323918</v>
       </c>
       <c r="E83" t="n">
         <v>25.94288334866243</v>
@@ -35641,7 +35641,7 @@
         <v>191.3136029182417</v>
       </c>
       <c r="D86" t="n">
-        <v>7.272450791640984</v>
+        <v>7.272450791640983</v>
       </c>
       <c r="E86" t="n">
         <v>26.3066204776716</v>
@@ -35679,7 +35679,7 @@
         <v>193.1329048905494</v>
       </c>
       <c r="D88" t="n">
-        <v>7.343162400456031</v>
+        <v>7.343162400456033</v>
       </c>
       <c r="E88" t="n">
         <v>26.30105319181764</v>
@@ -35698,7 +35698,7 @@
         <v>189.6053556316484</v>
       </c>
       <c r="D89" t="n">
-        <v>7.2061314812625</v>
+        <v>7.206131481262501</v>
       </c>
       <c r="E89" t="n">
         <v>26.311670294202</v>
@@ -35736,7 +35736,7 @@
         <v>129.6172607854945</v>
       </c>
       <c r="D91" t="n">
-        <v>4.906957553158348</v>
+        <v>4.906957553158349</v>
       </c>
       <c r="E91" t="n">
         <v>26.41499531661258</v>
@@ -35796,7 +35796,7 @@
         <v>3.229121460199138</v>
       </c>
       <c r="E94" t="n">
-        <v>26.44217382714826</v>
+        <v>26.44217382714825</v>
       </c>
     </row>
     <row r="95">
@@ -35831,10 +35831,10 @@
         <v>86.60890223076919</v>
       </c>
       <c r="D96" t="n">
-        <v>3.275465241517671</v>
+        <v>3.275465241517672</v>
       </c>
       <c r="E96" t="n">
-        <v>26.44171006090096</v>
+        <v>26.44171006090095</v>
       </c>
     </row>
     <row r="97">

</xml_diff>

<commit_message>
UI fixes, smoothed emission curves, corrected R2 values, and AI feedback training
- Fix time format: 24-hour to 12-hour AM/PM on hourly (R1) charts
- Correct R2 annual values by multiplying daily totals by 365
- Add vehicle type names to chart tooltips instead of tract IDs
- Improve x-axis layout: larger labels, tick marks, spacing, remove redundant Month label
- Add post-processing smoothing (Savitzky-Golay + Gaussian) to emission prediction curves
- Add AI feedback loop training script (train_with_feedback.py) for iterative model improvement
- Regenerate pregenerated JSON files and R1/R2 data with corrected values
- Update ML models for GA with feedback-loop-retrained weights

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/Combined_sheet_output_speed/GA/GA_2024.xlsx
+++ b/backend/Combined_sheet_output_speed/GA/GA_2024.xlsx
@@ -1,32 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="tract=13121001001" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="tract=13121001002" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="tract=13121001201" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="tract=13121001202" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="tract=13121001800" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="tract=13121001900" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="tract=13121002100" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="tract=13121002600" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="tract=13121002800" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="tract=13121003500" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="tract=13121003600" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="tract=13121003800" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="tract=13121004300" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="tract=13121004400" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="tract=13121004800" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="tract=13121004900" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="tract=13121005800" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="tract=13121011800" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="tract=13121011900" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="tract=13121012000" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001001" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001002" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001201" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001202" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001800" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121001900" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121002100" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121002600" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121002800" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121003500" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121003600" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121003800" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121004300" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121004400" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121004800" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121004900" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121005800" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121011800" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121011900" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tract=13121012000" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4069,10 +4069,10 @@
         <v>196.2035105142857</v>
       </c>
       <c r="D93" t="n">
-        <v>5.691074737075248</v>
+        <v>5.691074737075247</v>
       </c>
       <c r="E93" t="n">
-        <v>34.47565171409406</v>
+        <v>34.47565171409407</v>
       </c>
     </row>
     <row r="94">
@@ -4493,7 +4493,7 @@
         <v>1.170435024901576</v>
       </c>
       <c r="E17" t="n">
-        <v>27.12030829661201</v>
+        <v>27.120308296612</v>
       </c>
     </row>
     <row r="18">
@@ -6070,10 +6070,10 @@
         <v>30.61020132263733</v>
       </c>
       <c r="D2" t="n">
-        <v>1.339637886661133</v>
+        <v>1.339637886661134</v>
       </c>
       <c r="E2" t="n">
-        <v>22.84960856021259</v>
+        <v>22.84960856021258</v>
       </c>
     </row>
     <row r="3">
@@ -6089,10 +6089,10 @@
         <v>30.8829702606593</v>
       </c>
       <c r="D3" t="n">
-        <v>1.351575467616795</v>
+        <v>1.351575467616796</v>
       </c>
       <c r="E3" t="n">
-        <v>22.84960847588821</v>
+        <v>22.8496084758882</v>
       </c>
     </row>
     <row r="4">
@@ -6146,7 +6146,7 @@
         <v>8.891330181098876</v>
       </c>
       <c r="D6" t="n">
-        <v>0.389124004159705</v>
+        <v>0.3891240041597052</v>
       </c>
       <c r="E6" t="n">
         <v>22.84960600233153</v>
@@ -6165,7 +6165,7 @@
         <v>8.553209237802173</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3743263406205204</v>
+        <v>0.3743263406205205</v>
       </c>
       <c r="E7" t="n">
         <v>22.84960557043227</v>
@@ -6184,7 +6184,7 @@
         <v>8.362770709450526</v>
       </c>
       <c r="D8" t="n">
-        <v>0.3659919108581624</v>
+        <v>0.3659919108581625</v>
       </c>
       <c r="E8" t="n">
         <v>22.84960530914974</v>
@@ -6203,7 +6203,7 @@
         <v>8.762165989450523</v>
       </c>
       <c r="D9" t="n">
-        <v>0.3834712095278112</v>
+        <v>0.3834712095278113</v>
       </c>
       <c r="E9" t="n">
         <v>22.84960584196099</v>
@@ -6225,7 +6225,7 @@
         <v>0.1491087224935169</v>
       </c>
       <c r="E10" t="n">
-        <v>22.84958673440881</v>
+        <v>22.84958673440879</v>
       </c>
     </row>
     <row r="11">
@@ -6241,10 +6241,10 @@
         <v>3.464937085714264</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1516411235056714</v>
+        <v>0.1516411235056715</v>
       </c>
       <c r="E11" t="n">
-        <v>22.84958727297134</v>
+        <v>22.84958727297133</v>
       </c>
     </row>
     <row r="12">
@@ -6263,7 +6263,7 @@
         <v>0.1536923880863102</v>
       </c>
       <c r="E12" t="n">
-        <v>22.84958769596347</v>
+        <v>22.84958769596348</v>
       </c>
     </row>
     <row r="13">
@@ -6282,7 +6282,7 @@
         <v>0.1483807001011803</v>
       </c>
       <c r="E13" t="n">
-        <v>22.84958657611714</v>
+        <v>22.84958657611713</v>
       </c>
     </row>
     <row r="14">
@@ -6298,7 +6298,7 @@
         <v>3.875575657582396</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1696124767085144</v>
+        <v>0.1696124767085145</v>
       </c>
       <c r="E14" t="n">
         <v>22.84959062441333</v>
@@ -6320,7 +6320,7 @@
         <v>0.1678531282467341</v>
       </c>
       <c r="E15" t="n">
-        <v>22.84959032867342</v>
+        <v>22.84959032867341</v>
       </c>
     </row>
     <row r="16">
@@ -6336,7 +6336,7 @@
         <v>3.767189516043935</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1648690215882371</v>
+        <v>0.164869021588237</v>
       </c>
       <c r="E16" t="n">
         <v>22.84958981228474</v>
@@ -6374,10 +6374,10 @@
         <v>10.7662046452747</v>
       </c>
       <c r="D18" t="n">
-        <v>0.4711767804384162</v>
+        <v>0.4711767804384164</v>
       </c>
       <c r="E18" t="n">
-        <v>22.84960781653345</v>
+        <v>22.84960781653344</v>
       </c>
     </row>
     <row r="19">
@@ -6393,7 +6393,7 @@
         <v>10.21891783912085</v>
       </c>
       <c r="D19" t="n">
-        <v>0.4472250954914167</v>
+        <v>0.4472250954914168</v>
       </c>
       <c r="E19" t="n">
         <v>22.84960737252942</v>
@@ -6412,10 +6412,10 @@
         <v>10.76738327208788</v>
       </c>
       <c r="D20" t="n">
-        <v>0.4712283623474754</v>
+        <v>0.4712283623474757</v>
       </c>
       <c r="E20" t="n">
-        <v>22.84960781742633</v>
+        <v>22.84960781742631</v>
       </c>
     </row>
     <row r="21">
@@ -6431,10 +6431,10 @@
         <v>11.09893384615382</v>
       </c>
       <c r="D21" t="n">
-        <v>0.4857384782130515</v>
+        <v>0.4857384782130518</v>
       </c>
       <c r="E21" t="n">
-        <v>22.84960805860983</v>
+        <v>22.84960805860982</v>
       </c>
     </row>
     <row r="22">
@@ -6450,10 +6450,10 @@
         <v>54.09432631780217</v>
       </c>
       <c r="D22" t="n">
-        <v>2.367408649358135</v>
+        <v>2.367408649358136</v>
       </c>
       <c r="E22" t="n">
-        <v>22.84959393574427</v>
+        <v>22.84959393574426</v>
       </c>
     </row>
     <row r="23">
@@ -6469,10 +6469,10 @@
         <v>53.07156695999997</v>
       </c>
       <c r="D23" t="n">
-        <v>2.32264804111807</v>
+        <v>2.322648041118071</v>
       </c>
       <c r="E23" t="n">
-        <v>22.84959495389259</v>
+        <v>22.84959495389258</v>
       </c>
     </row>
     <row r="24">
@@ -6491,7 +6491,7 @@
         <v>2.409087392318296</v>
       </c>
       <c r="E24" t="n">
-        <v>22.84959294687103</v>
+        <v>22.84959294687102</v>
       </c>
     </row>
     <row r="25">
@@ -6526,10 +6526,10 @@
         <v>138.4873043960439</v>
       </c>
       <c r="D26" t="n">
-        <v>6.061046644566486</v>
+        <v>6.061046644566487</v>
       </c>
       <c r="E26" t="n">
-        <v>22.84874420496217</v>
+        <v>22.84874420496216</v>
       </c>
     </row>
     <row r="27">
@@ -6545,10 +6545,10 @@
         <v>139.7071534443956</v>
       </c>
       <c r="D27" t="n">
-        <v>6.114447461896395</v>
+        <v>6.114447461896398</v>
       </c>
       <c r="E27" t="n">
-        <v>22.84869635645957</v>
+        <v>22.84869635645956</v>
       </c>
     </row>
     <row r="28">
@@ -6564,10 +6564,10 @@
         <v>146.5498341824176</v>
       </c>
       <c r="D28" t="n">
-        <v>6.414015943449161</v>
+        <v>6.414015943449163</v>
       </c>
       <c r="E28" t="n">
-        <v>22.84837385415196</v>
+        <v>22.84837385415195</v>
       </c>
     </row>
     <row r="29">
@@ -6583,7 +6583,7 @@
         <v>161.3237490065934</v>
       </c>
       <c r="D29" t="n">
-        <v>7.060977310917817</v>
+        <v>7.060977310917818</v>
       </c>
       <c r="E29" t="n">
         <v>22.8472266519185</v>
@@ -6602,10 +6602,10 @@
         <v>223.4656607881318</v>
       </c>
       <c r="D30" t="n">
-        <v>9.797117149620167</v>
+        <v>9.797117149620169</v>
       </c>
       <c r="E30" t="n">
-        <v>22.80932823149875</v>
+        <v>22.80932823149874</v>
       </c>
     </row>
     <row r="31">
@@ -6621,7 +6621,7 @@
         <v>227.0606436593406</v>
       </c>
       <c r="D31" t="n">
-        <v>9.957931729957526</v>
+        <v>9.957931729957529</v>
       </c>
       <c r="E31" t="n">
         <v>22.80198838642862</v>
@@ -6643,7 +6643,7 @@
         <v>10.03690710232164</v>
       </c>
       <c r="E32" t="n">
-        <v>22.79791092562209</v>
+        <v>22.79791092562208</v>
       </c>
     </row>
     <row r="33">
@@ -6659,10 +6659,10 @@
         <v>229.7645977292308</v>
       </c>
       <c r="D33" t="n">
-        <v>10.07934938515903</v>
+        <v>10.07934938515904</v>
       </c>
       <c r="E33" t="n">
-        <v>22.79557826098768</v>
+        <v>22.79557826098767</v>
       </c>
     </row>
     <row r="34">
@@ -6678,10 +6678,10 @@
         <v>263.2762170738461</v>
       </c>
       <c r="D34" t="n">
-        <v>11.66041180274352</v>
+        <v>11.66041180274353</v>
       </c>
       <c r="E34" t="n">
-        <v>22.57863800418276</v>
+        <v>22.57863800418275</v>
       </c>
     </row>
     <row r="35">
@@ -6700,7 +6700,7 @@
         <v>12.01094184081939</v>
       </c>
       <c r="E35" t="n">
-        <v>22.46953243511504</v>
+        <v>22.46953243511503</v>
       </c>
     </row>
     <row r="36">
@@ -6716,10 +6716,10 @@
         <v>266.8434463727472</v>
       </c>
       <c r="D36" t="n">
-        <v>11.846654189603</v>
+        <v>11.84665418960301</v>
       </c>
       <c r="E36" t="n">
-        <v>22.52479409814608</v>
+        <v>22.52479409814607</v>
       </c>
     </row>
     <row r="37">
@@ -6754,10 +6754,10 @@
         <v>275.7965023806593</v>
       </c>
       <c r="D38" t="n">
-        <v>12.35190426487596</v>
+        <v>12.35190426487597</v>
       </c>
       <c r="E38" t="n">
-        <v>22.32825777033569</v>
+        <v>22.32825777033568</v>
       </c>
     </row>
     <row r="39">
@@ -6773,10 +6773,10 @@
         <v>271.9631481771428</v>
       </c>
       <c r="D39" t="n">
-        <v>12.12739822235165</v>
+        <v>12.12739822235166</v>
       </c>
       <c r="E39" t="n">
-        <v>22.42551478815097</v>
+        <v>22.42551478815096</v>
       </c>
     </row>
     <row r="40">
@@ -6814,7 +6814,7 @@
         <v>11.98618959695453</v>
       </c>
       <c r="E41" t="n">
-        <v>22.4783564237574</v>
+        <v>22.47835642375739</v>
       </c>
     </row>
     <row r="42">
@@ -6871,7 +6871,7 @@
         <v>13.20000053719058</v>
       </c>
       <c r="E44" t="n">
-        <v>21.79273481071968</v>
+        <v>21.79273481071967</v>
       </c>
     </row>
     <row r="45">
@@ -6890,7 +6890,7 @@
         <v>13.27723237766576</v>
       </c>
       <c r="E45" t="n">
-        <v>21.73017792834329</v>
+        <v>21.73017792834328</v>
       </c>
     </row>
     <row r="46">
@@ -6906,10 +6906,10 @@
         <v>313.1479132272528</v>
       </c>
       <c r="D46" t="n">
-        <v>15.64101465240685</v>
+        <v>15.64101465240686</v>
       </c>
       <c r="E46" t="n">
-        <v>20.02094622288877</v>
+        <v>20.02094622288876</v>
       </c>
     </row>
     <row r="47">
@@ -6928,7 +6928,7 @@
         <v>15.74819828987271</v>
       </c>
       <c r="E47" t="n">
-        <v>19.95269772843421</v>
+        <v>19.9526977284342</v>
       </c>
     </row>
     <row r="48">
@@ -6944,10 +6944,10 @@
         <v>314.7991741450549</v>
       </c>
       <c r="D48" t="n">
-        <v>15.80640289460823</v>
+        <v>15.80640289460824</v>
       </c>
       <c r="E48" t="n">
-        <v>19.91592750381157</v>
+        <v>19.91592750381156</v>
       </c>
     </row>
     <row r="49">
@@ -6963,10 +6963,10 @@
         <v>314.3879723986813</v>
       </c>
       <c r="D49" t="n">
-        <v>15.80640289460823</v>
+        <v>15.80640289460824</v>
       </c>
       <c r="E49" t="n">
-        <v>19.88991261926666</v>
+        <v>19.88991261926665</v>
       </c>
     </row>
     <row r="50">
@@ -6982,10 +6982,10 @@
         <v>359.3116791296703</v>
       </c>
       <c r="D50" t="n">
-        <v>20.64637778088954</v>
+        <v>20.64637778088955</v>
       </c>
       <c r="E50" t="n">
-        <v>17.40313399972039</v>
+        <v>17.40313399972038</v>
       </c>
     </row>
     <row r="51">
@@ -7001,10 +7001,10 @@
         <v>358.0589865520879</v>
       </c>
       <c r="D51" t="n">
-        <v>20.64637778088954</v>
+        <v>20.64637778088955</v>
       </c>
       <c r="E51" t="n">
-        <v>17.34246027811766</v>
+        <v>17.34246027811765</v>
       </c>
     </row>
     <row r="52">
@@ -7020,10 +7020,10 @@
         <v>357.6618475345055</v>
       </c>
       <c r="D52" t="n">
-        <v>20.64637778088954</v>
+        <v>20.64637778088955</v>
       </c>
       <c r="E52" t="n">
-        <v>17.32322499036903</v>
+        <v>17.32322499036902</v>
       </c>
     </row>
     <row r="53">
@@ -7039,10 +7039,10 @@
         <v>355.9815260993406</v>
       </c>
       <c r="D53" t="n">
-        <v>20.64637778088954</v>
+        <v>20.64637778088955</v>
       </c>
       <c r="E53" t="n">
-        <v>17.24183921640919</v>
+        <v>17.24183921640918</v>
       </c>
     </row>
     <row r="54">
@@ -7058,10 +7058,10 @@
         <v>349.8871248712088</v>
       </c>
       <c r="D54" t="n">
-        <v>20.64637778088954</v>
+        <v>20.64637778088955</v>
       </c>
       <c r="E54" t="n">
-        <v>16.94665905004738</v>
+        <v>16.94665905004737</v>
       </c>
     </row>
     <row r="55">
@@ -7077,10 +7077,10 @@
         <v>352.418698829011</v>
       </c>
       <c r="D55" t="n">
-        <v>20.94622832107846</v>
+        <v>20.94622832107848</v>
       </c>
       <c r="E55" t="n">
-        <v>16.82492396372704</v>
+        <v>16.82492396372703</v>
       </c>
     </row>
     <row r="56">
@@ -7096,10 +7096,10 @@
         <v>349.4623142624176</v>
       </c>
       <c r="D56" t="n">
-        <v>20.94622832107846</v>
+        <v>20.94622832107848</v>
       </c>
       <c r="E56" t="n">
-        <v>16.68378234523249</v>
+        <v>16.68378234523248</v>
       </c>
     </row>
     <row r="57">
@@ -7115,10 +7115,10 @@
         <v>349.6339589208791</v>
       </c>
       <c r="D57" t="n">
-        <v>20.9668096027182</v>
+        <v>20.96680960271821</v>
       </c>
       <c r="E57" t="n">
-        <v>16.67559183041141</v>
+        <v>16.6755918304114</v>
       </c>
     </row>
     <row r="58">
@@ -7134,10 +7134,10 @@
         <v>355.2095671213186</v>
       </c>
       <c r="D58" t="n">
-        <v>21.64085647713941</v>
+        <v>21.64085647713943</v>
       </c>
       <c r="E58" t="n">
-        <v>16.41384052874934</v>
+        <v>16.41384052874933</v>
       </c>
     </row>
     <row r="59">
@@ -7153,10 +7153,10 @@
         <v>355.5885918804395</v>
       </c>
       <c r="D59" t="n">
-        <v>21.68706467281215</v>
+        <v>21.68706467281216</v>
       </c>
       <c r="E59" t="n">
-        <v>16.39634488323452</v>
+        <v>16.39634488323451</v>
       </c>
     </row>
     <row r="60">
@@ -7172,10 +7172,10 @@
         <v>348.4196655771428</v>
       </c>
       <c r="D60" t="n">
-        <v>21.68706467281215</v>
+        <v>21.68706467281216</v>
       </c>
       <c r="E60" t="n">
-        <v>16.0657825682577</v>
+        <v>16.06578256825769</v>
       </c>
     </row>
     <row r="61">
@@ -7191,10 +7191,10 @@
         <v>349.3192596210989</v>
       </c>
       <c r="D61" t="n">
-        <v>21.79919806974794</v>
+        <v>21.79919806974796</v>
       </c>
       <c r="E61" t="n">
-        <v>16.02440871923038</v>
+        <v>16.02440871923037</v>
       </c>
     </row>
     <row r="62">
@@ -7210,10 +7210,10 @@
         <v>356.8486793907691</v>
       </c>
       <c r="D62" t="n">
-        <v>22.74906979780212</v>
+        <v>22.74906979780213</v>
       </c>
       <c r="E62" t="n">
-        <v>15.68629761843035</v>
+        <v>15.68629761843034</v>
       </c>
     </row>
     <row r="63">
@@ -7229,10 +7229,10 @@
         <v>358.3253799745054</v>
       </c>
       <c r="D63" t="n">
-        <v>22.9377384102348</v>
+        <v>22.93773841023481</v>
       </c>
       <c r="E63" t="n">
-        <v>15.6216525607695</v>
+        <v>15.62165256076949</v>
       </c>
     </row>
     <row r="64">
@@ -7248,10 +7248,10 @@
         <v>354.358451233846</v>
       </c>
       <c r="D64" t="n">
-        <v>22.9377384102348</v>
+        <v>22.93773841023481</v>
       </c>
       <c r="E64" t="n">
-        <v>15.4487092361177</v>
+        <v>15.44870923611769</v>
       </c>
     </row>
     <row r="65">
@@ -7267,10 +7267,10 @@
         <v>352.5632267538461</v>
       </c>
       <c r="D65" t="n">
-        <v>22.9377384102348</v>
+        <v>22.93773841023481</v>
       </c>
       <c r="E65" t="n">
-        <v>15.37044413221369</v>
+        <v>15.37044413221368</v>
       </c>
     </row>
     <row r="66">
@@ -7286,10 +7286,10 @@
         <v>373.7397727279121</v>
       </c>
       <c r="D66" t="n">
-        <v>25.77598114035739</v>
+        <v>25.77598114035741</v>
       </c>
       <c r="E66" t="n">
-        <v>14.4995362423954</v>
+        <v>14.49953624239538</v>
       </c>
     </row>
     <row r="67">
@@ -7305,10 +7305,10 @@
         <v>373.2558834501098</v>
       </c>
       <c r="D67" t="n">
-        <v>25.77598114035738</v>
+        <v>25.7759811403574</v>
       </c>
       <c r="E67" t="n">
-        <v>14.48076336716836</v>
+        <v>14.48076336716835</v>
       </c>
     </row>
     <row r="68">
@@ -7324,10 +7324,10 @@
         <v>373.7905071468131</v>
       </c>
       <c r="D68" t="n">
-        <v>25.84987318051506</v>
+        <v>25.84987318051508</v>
       </c>
       <c r="E68" t="n">
-        <v>14.46005187478314</v>
+        <v>14.46005187478313</v>
       </c>
     </row>
     <row r="69">
@@ -7343,10 +7343,10 @@
         <v>375.2396454474725</v>
       </c>
       <c r="D69" t="n">
-        <v>26.05069505525815</v>
+        <v>26.05069505525817</v>
       </c>
       <c r="E69" t="n">
-        <v>14.40420858835139</v>
+        <v>14.40420858835138</v>
       </c>
     </row>
     <row r="70">
@@ -7362,10 +7362,10 @@
         <v>370.5674071740658</v>
       </c>
       <c r="D70" t="n">
-        <v>25.40600146870595</v>
+        <v>25.40600146870596</v>
       </c>
       <c r="E70" t="n">
-        <v>14.58582168589242</v>
+        <v>14.58582168589241</v>
       </c>
     </row>
     <row r="71">
@@ -7381,10 +7381,10 @@
         <v>370.6651749810989</v>
       </c>
       <c r="D71" t="n">
-        <v>25.40600146870595</v>
+        <v>25.40600146870596</v>
       </c>
       <c r="E71" t="n">
-        <v>14.58966990290341</v>
+        <v>14.5896699029034</v>
       </c>
     </row>
     <row r="72">
@@ -7400,10 +7400,10 @@
         <v>374.37187908</v>
       </c>
       <c r="D72" t="n">
-        <v>25.40600146870595</v>
+        <v>25.40600146870596</v>
       </c>
       <c r="E72" t="n">
-        <v>14.73556866243339</v>
+        <v>14.73556866243338</v>
       </c>
     </row>
     <row r="73">
@@ -7419,10 +7419,10 @@
         <v>374.6524932527472</v>
       </c>
       <c r="D73" t="n">
-        <v>25.40600146870595</v>
+        <v>25.40600146870596</v>
       </c>
       <c r="E73" t="n">
-        <v>14.74661385477083</v>
+        <v>14.74661385477082</v>
       </c>
     </row>
     <row r="74">
@@ -7441,7 +7441,7 @@
         <v>20.97430976998552</v>
       </c>
       <c r="E74" t="n">
-        <v>16.22992932939863</v>
+        <v>16.22992932939862</v>
       </c>
     </row>
     <row r="75">
@@ -7457,10 +7457,10 @@
         <v>337.3097902246154</v>
       </c>
       <c r="D75" t="n">
-        <v>20.59382214415265</v>
+        <v>20.59382214415266</v>
       </c>
       <c r="E75" t="n">
-        <v>16.3791737086741</v>
+        <v>16.37917370867409</v>
       </c>
     </row>
     <row r="76">
@@ -7476,10 +7476,10 @@
         <v>337.4643875670329</v>
       </c>
       <c r="D76" t="n">
-        <v>20.59382214415265</v>
+        <v>20.59382214415266</v>
       </c>
       <c r="E76" t="n">
-        <v>16.3866806853458</v>
+        <v>16.38668068534579</v>
       </c>
     </row>
     <row r="77">
@@ -7495,10 +7495,10 @@
         <v>337.4051128562637</v>
       </c>
       <c r="D77" t="n">
-        <v>20.58658828072593</v>
+        <v>20.58658828072594</v>
       </c>
       <c r="E77" t="n">
-        <v>16.38955946732355</v>
+        <v>16.38955946732354</v>
       </c>
     </row>
     <row r="78">
@@ -7517,7 +7517,7 @@
         <v>12.59805847935922</v>
       </c>
       <c r="E78" t="n">
-        <v>22.20122132749056</v>
+        <v>22.20122132749055</v>
       </c>
     </row>
     <row r="79">
@@ -7536,7 +7536,7 @@
         <v>12.51603357187028</v>
       </c>
       <c r="E79" t="n">
-        <v>22.24603320795041</v>
+        <v>22.2460332079504</v>
       </c>
     </row>
     <row r="80">
@@ -7555,7 +7555,7 @@
         <v>12.42511964104743</v>
       </c>
       <c r="E80" t="n">
-        <v>22.29278342953694</v>
+        <v>22.29278342953693</v>
       </c>
     </row>
     <row r="81">
@@ -7574,7 +7574,7 @@
         <v>12.29512509585927</v>
       </c>
       <c r="E81" t="n">
-        <v>22.35446698484215</v>
+        <v>22.35446698484214</v>
       </c>
     </row>
     <row r="82">
@@ -7590,10 +7590,10 @@
         <v>213.7335229516484</v>
       </c>
       <c r="D82" t="n">
-        <v>9.364444672973406</v>
+        <v>9.364444672973407</v>
       </c>
       <c r="E82" t="n">
-        <v>22.8239399575398</v>
+        <v>22.82393995753979</v>
       </c>
     </row>
     <row r="83">
@@ -7609,10 +7609,10 @@
         <v>212.4219156672527</v>
       </c>
       <c r="D83" t="n">
-        <v>9.306364248388739</v>
+        <v>9.306364248388743</v>
       </c>
       <c r="E83" t="n">
-        <v>22.82544611382801</v>
+        <v>22.825446113828</v>
       </c>
     </row>
     <row r="84">
@@ -7628,10 +7628,10 @@
         <v>213.8133749182417</v>
       </c>
       <c r="D84" t="n">
-        <v>9.367982155594127</v>
+        <v>9.367982155594131</v>
       </c>
       <c r="E84" t="n">
-        <v>22.8238452387062</v>
+        <v>22.82384523870619</v>
       </c>
     </row>
     <row r="85">
@@ -7647,10 +7647,10 @@
         <v>213.4275219652748</v>
       </c>
       <c r="D85" t="n">
-        <v>9.350890282891452</v>
+        <v>9.350890282891458</v>
       </c>
       <c r="E85" t="n">
-        <v>22.82429966649972</v>
+        <v>22.8242996664997</v>
       </c>
     </row>
     <row r="86">
@@ -7666,10 +7666,10 @@
         <v>157.1992609107692</v>
       </c>
       <c r="D86" t="n">
-        <v>6.880332110156038</v>
+        <v>6.880332110156041</v>
       </c>
       <c r="E86" t="n">
-        <v>22.84762688689516</v>
+        <v>22.84762688689515</v>
       </c>
     </row>
     <row r="87">
@@ -7685,7 +7685,7 @@
         <v>156.2733735085714</v>
       </c>
       <c r="D87" t="n">
-        <v>6.839783698075112</v>
+        <v>6.839783698075113</v>
       </c>
       <c r="E87" t="n">
         <v>22.84770694613496</v>
@@ -7704,10 +7704,10 @@
         <v>156.2389913485714</v>
       </c>
       <c r="D88" t="n">
-        <v>6.838277986665286</v>
+        <v>6.838277986665289</v>
       </c>
       <c r="E88" t="n">
-        <v>22.8477098552061</v>
+        <v>22.84770985520609</v>
       </c>
     </row>
     <row r="89">
@@ -7723,7 +7723,7 @@
         <v>156.7579186351648</v>
       </c>
       <c r="D89" t="n">
-        <v>6.861003758597583</v>
+        <v>6.861003758597586</v>
       </c>
       <c r="E89" t="n">
         <v>22.84766546567331</v>
@@ -7742,10 +7742,10 @@
         <v>99.50524790769229</v>
       </c>
       <c r="D90" t="n">
-        <v>4.354819408693424</v>
+        <v>4.354819408693426</v>
       </c>
       <c r="E90" t="n">
-        <v>22.84945449380801</v>
+        <v>22.849454493808</v>
       </c>
     </row>
     <row r="91">
@@ -7761,7 +7761,7 @@
         <v>100.3838488496703</v>
       </c>
       <c r="D91" t="n">
-        <v>4.393272326514579</v>
+        <v>4.39327232651458</v>
       </c>
       <c r="E91" t="n">
         <v>22.84944829024752</v>
@@ -7780,10 +7780,10 @@
         <v>99.95495938417579</v>
       </c>
       <c r="D92" t="n">
-        <v>4.374501508275402</v>
+        <v>4.374501508275404</v>
       </c>
       <c r="E92" t="n">
-        <v>22.84945134779069</v>
+        <v>22.84945134779068</v>
       </c>
     </row>
     <row r="93">
@@ -7799,10 +7799,10 @@
         <v>101.8805136131868</v>
       </c>
       <c r="D93" t="n">
-        <v>4.458775630484695</v>
+        <v>4.458775630484696</v>
       </c>
       <c r="E93" t="n">
-        <v>22.84943716760016</v>
+        <v>22.84943716760015</v>
       </c>
     </row>
     <row r="94">
@@ -7818,10 +7818,10 @@
         <v>62.4277858140659</v>
       </c>
       <c r="D94" t="n">
-        <v>2.732119168847426</v>
+        <v>2.732119168847428</v>
       </c>
       <c r="E94" t="n">
-        <v>22.84958376848611</v>
+        <v>22.8495837684861</v>
       </c>
     </row>
     <row r="95">
@@ -7837,7 +7837,7 @@
         <v>62.82371174901096</v>
       </c>
       <c r="D95" t="n">
-        <v>2.749446728368237</v>
+        <v>2.749446728368238</v>
       </c>
       <c r="E95" t="n">
         <v>22.8495831909775</v>
@@ -7875,10 +7875,10 @@
         <v>64.24512974505491</v>
       </c>
       <c r="D97" t="n">
-        <v>2.811654605017022</v>
+        <v>2.811654605017023</v>
       </c>
       <c r="E97" t="n">
-        <v>22.84958103688059</v>
+        <v>22.84958103688058</v>
       </c>
     </row>
   </sheetData>
@@ -8201,7 +8201,7 @@
         <v>29.73550933450547</v>
       </c>
       <c r="D16" t="n">
-        <v>1.36757739048477</v>
+        <v>1.367577390484771</v>
       </c>
       <c r="E16" t="n">
         <v>21.74320045168706</v>
@@ -9898,7 +9898,7 @@
         <v>1.69278012320381</v>
       </c>
       <c r="E7" t="n">
-        <v>50.80135384759658</v>
+        <v>50.80135384759659</v>
       </c>
     </row>
     <row r="8">
@@ -12520,7 +12520,7 @@
         <v>886.1867469217582</v>
       </c>
       <c r="D47" t="n">
-        <v>24.5146043949178</v>
+        <v>24.51460439491779</v>
       </c>
       <c r="E47" t="n">
         <v>36.14933908970102</v>
@@ -12558,10 +12558,10 @@
         <v>882.9076835617583</v>
       </c>
       <c r="D49" t="n">
-        <v>23.02039947266763</v>
+        <v>23.02039947266762</v>
       </c>
       <c r="E49" t="n">
-        <v>38.35327378267455</v>
+        <v>38.35327378267456</v>
       </c>
     </row>
     <row r="50">
@@ -12710,10 +12710,10 @@
         <v>956.9201780650548</v>
       </c>
       <c r="D57" t="n">
-        <v>26.48066679529901</v>
+        <v>26.48066679529898</v>
       </c>
       <c r="E57" t="n">
-        <v>36.13655900216729</v>
+        <v>36.13655900216732</v>
       </c>
     </row>
     <row r="58">
@@ -13549,7 +13549,7 @@
         <v>159.970558294945</v>
       </c>
       <c r="D3" t="n">
-        <v>3.097782632988745</v>
+        <v>3.097782632988746</v>
       </c>
       <c r="E3" t="n">
         <v>51.64034318980126</v>
@@ -14312,7 +14312,7 @@
         <v>20.6195859462152</v>
       </c>
       <c r="E43" t="n">
-        <v>29.67954999234207</v>
+        <v>29.67954999234206</v>
       </c>
     </row>
     <row r="44">
@@ -14404,10 +14404,10 @@
         <v>635.4690135942856</v>
       </c>
       <c r="D48" t="n">
-        <v>20.62770722371686</v>
+        <v>20.62770722371687</v>
       </c>
       <c r="E48" t="n">
-        <v>30.80657519046277</v>
+        <v>30.80657519046276</v>
       </c>
     </row>
     <row r="49">
@@ -15398,7 +15398,7 @@
         <v>1.820265680860277</v>
       </c>
       <c r="E2" t="n">
-        <v>44.72506916959536</v>
+        <v>44.72506916959535</v>
       </c>
     </row>
     <row r="3">
@@ -15547,10 +15547,10 @@
         <v>39.26279422681316</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8782236739649278</v>
+        <v>0.878223673964928</v>
       </c>
       <c r="E10" t="n">
-        <v>44.70705515094226</v>
+        <v>44.70705515094225</v>
       </c>
     </row>
     <row r="11">
@@ -15585,10 +15585,10 @@
         <v>39.06507957890107</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8738130900206208</v>
+        <v>0.8738130900206209</v>
       </c>
       <c r="E12" t="n">
-        <v>44.70644812379635</v>
+        <v>44.70644812379634</v>
       </c>
     </row>
     <row r="13">
@@ -15642,10 +15642,10 @@
         <v>40.99139777670326</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9167877245148059</v>
+        <v>0.9167877245148061</v>
       </c>
       <c r="E15" t="n">
-        <v>44.71198368018862</v>
+        <v>44.71198368018861</v>
       </c>
     </row>
     <row r="16">
@@ -15661,7 +15661,7 @@
         <v>40.48648212923074</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9055228781791316</v>
+        <v>0.9055228781791317</v>
       </c>
       <c r="E16" t="n">
         <v>44.71061207270972</v>
@@ -15680,10 +15680,10 @@
         <v>42.27254017186809</v>
       </c>
       <c r="D17" t="n">
-        <v>0.9453723377361275</v>
+        <v>0.9453723377361274</v>
       </c>
       <c r="E17" t="n">
-        <v>44.71522857660259</v>
+        <v>44.7152285766026</v>
       </c>
     </row>
     <row r="18">
@@ -15927,7 +15927,7 @@
         <v>326.1173515885714</v>
       </c>
       <c r="D30" t="n">
-        <v>8.018276470510139</v>
+        <v>8.018276470510138</v>
       </c>
       <c r="E30" t="n">
         <v>40.67175193920735</v>
@@ -15946,10 +15946,10 @@
         <v>324.2464074646153</v>
       </c>
       <c r="D31" t="n">
-        <v>7.946580022795576</v>
+        <v>7.946580022795573</v>
       </c>
       <c r="E31" t="n">
-        <v>40.80326461628542</v>
+        <v>40.80326461628543</v>
       </c>
     </row>
     <row r="32">
@@ -15965,10 +15965,10 @@
         <v>319.2360458716483</v>
       </c>
       <c r="D32" t="n">
-        <v>7.761683856325791</v>
+        <v>7.76168385632579</v>
       </c>
       <c r="E32" t="n">
-        <v>41.12974088882403</v>
+        <v>41.12974088882404</v>
       </c>
     </row>
     <row r="33">
@@ -15984,10 +15984,10 @@
         <v>326.00526204</v>
       </c>
       <c r="D33" t="n">
-        <v>8.013936827213081</v>
+        <v>8.01393682721308</v>
       </c>
       <c r="E33" t="n">
-        <v>40.67978935558583</v>
+        <v>40.67978935558584</v>
       </c>
     </row>
     <row r="34">
@@ -16003,10 +16003,10 @@
         <v>355.4561805243956</v>
       </c>
       <c r="D34" t="n">
-        <v>9.490166662544075</v>
+        <v>9.49016666254407</v>
       </c>
       <c r="E34" t="n">
-        <v>37.45520949882947</v>
+        <v>37.45520949882949</v>
       </c>
     </row>
     <row r="35">
@@ -16022,10 +16022,10 @@
         <v>359.0433217252747</v>
       </c>
       <c r="D35" t="n">
-        <v>9.759111073797213</v>
+        <v>9.759111073797207</v>
       </c>
       <c r="E35" t="n">
-        <v>36.79057641728153</v>
+        <v>36.79057641728155</v>
       </c>
     </row>
     <row r="36">
@@ -16041,7 +16041,7 @@
         <v>361.4715793002197</v>
       </c>
       <c r="D36" t="n">
-        <v>9.965435595615281</v>
+        <v>9.965435595615279</v>
       </c>
       <c r="E36" t="n">
         <v>36.27253177565711</v>
@@ -16063,7 +16063,7 @@
         <v>10.08348261519677</v>
       </c>
       <c r="E37" t="n">
-        <v>35.97391999097246</v>
+        <v>35.97391999097248</v>
       </c>
     </row>
     <row r="38">
@@ -16079,10 +16079,10 @@
         <v>368.2786968751648</v>
       </c>
       <c r="D38" t="n">
-        <v>10.72016529063768</v>
+        <v>10.72016529063767</v>
       </c>
       <c r="E38" t="n">
-        <v>34.35382635347948</v>
+        <v>34.35382635347952</v>
       </c>
     </row>
     <row r="39">
@@ -16098,10 +16098,10 @@
         <v>367.3143270698901</v>
       </c>
       <c r="D39" t="n">
-        <v>10.59024266086115</v>
+        <v>10.59024266086114</v>
       </c>
       <c r="E39" t="n">
-        <v>34.68422196097459</v>
+        <v>34.6842219609746</v>
       </c>
     </row>
     <row r="40">
@@ -16117,10 +16117,10 @@
         <v>366.5890842487912</v>
       </c>
       <c r="D40" t="n">
-        <v>10.49895456276678</v>
+        <v>10.49895456276677</v>
       </c>
       <c r="E40" t="n">
-        <v>34.91672261815984</v>
+        <v>34.91672261815987</v>
       </c>
     </row>
     <row r="41">
@@ -16139,7 +16139,7 @@
         <v>10.29912897066958</v>
       </c>
       <c r="E41" t="n">
-        <v>35.42584617606715</v>
+        <v>35.42584617606716</v>
       </c>
     </row>
     <row r="42">
@@ -16177,7 +16177,7 @@
         <v>11.659698346108</v>
       </c>
       <c r="E43" t="n">
-        <v>33.200155688851</v>
+        <v>33.20015568885101</v>
       </c>
     </row>
     <row r="44">
@@ -16196,7 +16196,7 @@
         <v>11.659698346108</v>
       </c>
       <c r="E44" t="n">
-        <v>33.17710941030693</v>
+        <v>33.17710941030694</v>
       </c>
     </row>
     <row r="45">
@@ -16212,10 +16212,10 @@
         <v>386.840043418022</v>
       </c>
       <c r="D45" t="n">
-        <v>11.65999709002232</v>
+        <v>11.65999709002231</v>
       </c>
       <c r="E45" t="n">
-        <v>33.176684387773</v>
+        <v>33.17668438777301</v>
       </c>
     </row>
     <row r="46">
@@ -16234,7 +16234,7 @@
         <v>12.98655619110549</v>
       </c>
       <c r="E46" t="n">
-        <v>31.43657348568708</v>
+        <v>31.43657348568709</v>
       </c>
     </row>
     <row r="47">
@@ -16272,7 +16272,7 @@
         <v>13.08933214593559</v>
       </c>
       <c r="E48" t="n">
-        <v>31.20644637664552</v>
+        <v>31.20644637664553</v>
       </c>
     </row>
     <row r="49">
@@ -16288,10 +16288,10 @@
         <v>410.8768778531868</v>
       </c>
       <c r="D49" t="n">
-        <v>13.2439423933353</v>
+        <v>13.24394239333529</v>
       </c>
       <c r="E49" t="n">
-        <v>31.02375906285661</v>
+        <v>31.02375906285662</v>
       </c>
     </row>
     <row r="50">
@@ -16842,7 +16842,7 @@
         <v>13.64106764145922</v>
       </c>
       <c r="E78" t="n">
-        <v>30.83453724442678</v>
+        <v>30.83453724442677</v>
       </c>
     </row>
     <row r="79">
@@ -16855,13 +16855,13 @@
         <v>375.7576008421977</v>
       </c>
       <c r="C79" t="n">
-        <v>401.1420841510562</v>
+        <v>401.1420841510563</v>
       </c>
       <c r="D79" t="n">
-        <v>12.40718393359743</v>
+        <v>12.40718393359744</v>
       </c>
       <c r="E79" t="n">
-        <v>32.33143687543819</v>
+        <v>32.33143687543817</v>
       </c>
     </row>
     <row r="80">
@@ -16874,13 +16874,13 @@
         <v>375.2319023920878</v>
       </c>
       <c r="C80" t="n">
-        <v>381.6681600577931</v>
+        <v>381.6681600577932</v>
       </c>
       <c r="D80" t="n">
-        <v>11.23178108011159</v>
+        <v>11.2317810801116</v>
       </c>
       <c r="E80" t="n">
-        <v>33.98108967184403</v>
+        <v>33.98108967184401</v>
       </c>
     </row>
     <row r="81">
@@ -16896,10 +16896,10 @@
         <v>370.9064916923076</v>
       </c>
       <c r="D81" t="n">
-        <v>11.1406893323284</v>
+        <v>11.14068933232838</v>
       </c>
       <c r="E81" t="n">
-        <v>33.29295707187523</v>
+        <v>33.29295707187526</v>
       </c>
     </row>
     <row r="82">
@@ -16915,10 +16915,10 @@
         <v>309.8524061221977</v>
       </c>
       <c r="D82" t="n">
-        <v>7.438362165073412</v>
+        <v>7.438362165073411</v>
       </c>
       <c r="E82" t="n">
-        <v>41.6559988940979</v>
+        <v>41.65599889409791</v>
       </c>
     </row>
     <row r="83">
@@ -16953,10 +16953,10 @@
         <v>306.6639413815385</v>
       </c>
       <c r="D84" t="n">
-        <v>7.334079404880689</v>
+        <v>7.334079404880686</v>
       </c>
       <c r="E84" t="n">
-        <v>41.81355620140403</v>
+        <v>41.81355620140405</v>
       </c>
     </row>
     <row r="85">
@@ -16972,10 +16972,10 @@
         <v>309.0563090571429</v>
       </c>
       <c r="D85" t="n">
-        <v>7.412088082434233</v>
+        <v>7.412088082434232</v>
       </c>
       <c r="E85" t="n">
-        <v>41.69625422956989</v>
+        <v>41.6962542295699</v>
       </c>
     </row>
     <row r="86">
@@ -17010,10 +17010,10 @@
         <v>242.9158202663736</v>
       </c>
       <c r="D87" t="n">
-        <v>5.562932831851892</v>
+        <v>5.562932831851891</v>
       </c>
       <c r="E87" t="n">
-        <v>43.66686199687715</v>
+        <v>43.66686199687716</v>
       </c>
     </row>
     <row r="88">
@@ -17032,7 +17032,7 @@
         <v>5.497454971511043</v>
       </c>
       <c r="E88" t="n">
-        <v>43.71020664956544</v>
+        <v>43.71020664956545</v>
       </c>
     </row>
     <row r="89">
@@ -17048,10 +17048,10 @@
         <v>237.8689248065933</v>
       </c>
       <c r="D89" t="n">
-        <v>5.437144224148089</v>
+        <v>5.437144224148088</v>
       </c>
       <c r="E89" t="n">
-        <v>43.74887165033101</v>
+        <v>43.74887165033102</v>
       </c>
     </row>
     <row r="90">
@@ -17086,10 +17086,10 @@
         <v>177.8669074312087</v>
       </c>
       <c r="D91" t="n">
-        <v>4.007682068430383</v>
+        <v>4.007682068430382</v>
       </c>
       <c r="E91" t="n">
-        <v>44.38149144422292</v>
+        <v>44.38149144422294</v>
       </c>
     </row>
     <row r="92">
@@ -17143,10 +17143,10 @@
         <v>126.6238148215384</v>
       </c>
       <c r="D94" t="n">
-        <v>2.837327583076174</v>
+        <v>2.837327583076175</v>
       </c>
       <c r="E94" t="n">
-        <v>44.62784472854396</v>
+        <v>44.62784472854395</v>
       </c>
     </row>
     <row r="95">
@@ -17162,10 +17162,10 @@
         <v>126.2645593885714</v>
       </c>
       <c r="D95" t="n">
-        <v>2.829204416427379</v>
+        <v>2.82920441642738</v>
       </c>
       <c r="E95" t="n">
-        <v>44.62899840514667</v>
+        <v>44.62899840514666</v>
       </c>
     </row>
     <row r="96">
@@ -17526,10 +17526,10 @@
         <v>18.621741661978</v>
       </c>
       <c r="D16" t="n">
-        <v>0.6757281054966087</v>
+        <v>0.6757281054966088</v>
       </c>
       <c r="E16" t="n">
-        <v>27.55803926239303</v>
+        <v>27.55803926239302</v>
       </c>
     </row>
     <row r="17">
@@ -23390,7 +23390,7 @@
         <v>14.73481664071972</v>
       </c>
       <c r="E30" t="n">
-        <v>44.91717488346737</v>
+        <v>44.91717488346736</v>
       </c>
     </row>
     <row r="31">
@@ -23580,7 +23580,7 @@
         <v>18.6983032232002</v>
       </c>
       <c r="E40" t="n">
-        <v>38.14473108690226</v>
+        <v>38.14473108690227</v>
       </c>
     </row>
     <row r="41">
@@ -23672,10 +23672,10 @@
         <v>753.9345874786814</v>
       </c>
       <c r="D45" t="n">
-        <v>24.65702128837261</v>
+        <v>24.65702128837262</v>
       </c>
       <c r="E45" t="n">
-        <v>30.57687214774035</v>
+        <v>30.57687214774034</v>
       </c>
     </row>
     <row r="46">
@@ -26645,7 +26645,7 @@
         <v>1.950953788585696</v>
       </c>
       <c r="E5" t="n">
-        <v>17.63168434334251</v>
+        <v>17.63168434334252</v>
       </c>
     </row>
     <row r="6">
@@ -26661,10 +26661,10 @@
         <v>18.82210584395602</v>
       </c>
       <c r="D6" t="n">
-        <v>1.067555721595734</v>
+        <v>1.067555721595735</v>
       </c>
       <c r="E6" t="n">
-        <v>17.63102896008237</v>
+        <v>17.63102896008236</v>
       </c>
     </row>
     <row r="7">
@@ -26737,7 +26737,7 @@
         <v>14.24225314021976</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8078363696900435</v>
+        <v>0.8078363696900437</v>
       </c>
       <c r="E10" t="n">
         <v>17.63012124062244</v>
@@ -26794,7 +26794,7 @@
         <v>13.94441224351646</v>
       </c>
       <c r="D13" t="n">
-        <v>0.7909463333715731</v>
+        <v>0.7909463333715732</v>
       </c>
       <c r="E13" t="n">
         <v>17.63003588887694</v>
@@ -26832,7 +26832,7 @@
         <v>14.93218111780217</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8469610931524456</v>
+        <v>0.8469610931524457</v>
       </c>
       <c r="E15" t="n">
         <v>17.63030349153772</v>
@@ -26851,7 +26851,7 @@
         <v>15.2575617230769</v>
       </c>
       <c r="D16" t="n">
-        <v>0.8654129685162603</v>
+        <v>0.8654129685162604</v>
       </c>
       <c r="E16" t="n">
         <v>17.6303825781994</v>
@@ -26870,7 +26870,7 @@
         <v>14.92485509670327</v>
       </c>
       <c r="D17" t="n">
-        <v>0.8465456452435166</v>
+        <v>0.8465456452435167</v>
       </c>
       <c r="E17" t="n">
         <v>17.63030166248153</v>
@@ -26930,7 +26930,7 @@
         <v>1.32257239082003</v>
       </c>
       <c r="E20" t="n">
-        <v>17.63146792285391</v>
+        <v>17.63146792285392</v>
       </c>
     </row>
     <row r="21">
@@ -26965,7 +26965,7 @@
         <v>54.4823416707692</v>
       </c>
       <c r="D22" t="n">
-        <v>3.090218557000249</v>
+        <v>3.090218557000248</v>
       </c>
       <c r="E22" t="n">
         <v>17.63057876516558</v>
@@ -27041,10 +27041,10 @@
         <v>137.6859652931868</v>
       </c>
       <c r="D26" t="n">
-        <v>7.823253140948955</v>
+        <v>7.823253140948957</v>
       </c>
       <c r="E26" t="n">
-        <v>17.59957946042963</v>
+        <v>17.59957946042962</v>
       </c>
     </row>
     <row r="27">
@@ -27079,7 +27079,7 @@
         <v>145.4823309665934</v>
       </c>
       <c r="D28" t="n">
-        <v>8.270022597790607</v>
+        <v>8.270022597790609</v>
       </c>
       <c r="E28" t="n">
         <v>17.59152762236224</v>
@@ -27098,7 +27098,7 @@
         <v>147.3403351463736</v>
       </c>
       <c r="D29" t="n">
-        <v>8.376680926737711</v>
+        <v>8.376680926737713</v>
       </c>
       <c r="E29" t="n">
         <v>17.58934552181339</v>
@@ -27155,7 +27155,7 @@
         <v>234.9429207718681</v>
       </c>
       <c r="D32" t="n">
-        <v>13.72902850525163</v>
+        <v>13.72902850525162</v>
       </c>
       <c r="E32" t="n">
         <v>17.11285839941244</v>
@@ -27326,7 +27326,7 @@
         <v>270.1830462395604</v>
       </c>
       <c r="D41" t="n">
-        <v>17.07102601785775</v>
+        <v>17.07102601785776</v>
       </c>
       <c r="E41" t="n">
         <v>15.82699516460966</v>
@@ -27345,7 +27345,7 @@
         <v>274.9312061393406</v>
       </c>
       <c r="D42" t="n">
-        <v>17.9054568036542</v>
+        <v>17.90545680365421</v>
       </c>
       <c r="E42" t="n">
         <v>15.3546044177567</v>
@@ -27364,10 +27364,10 @@
         <v>275.4136197573625</v>
       </c>
       <c r="D43" t="n">
-        <v>18.00772225973985</v>
+        <v>18.00772225973986</v>
       </c>
       <c r="E43" t="n">
-        <v>15.29419522274114</v>
+        <v>15.29419522274113</v>
       </c>
     </row>
     <row r="44">
@@ -27386,7 +27386,7 @@
         <v>18.17743058766879</v>
       </c>
       <c r="E44" t="n">
-        <v>15.19303261609004</v>
+        <v>15.19303261609005</v>
       </c>
     </row>
     <row r="45">
@@ -27402,7 +27402,7 @@
         <v>279.3751460624176</v>
       </c>
       <c r="D45" t="n">
-        <v>19.08060323837802</v>
+        <v>19.08060323837801</v>
       </c>
       <c r="E45" t="n">
         <v>14.64184033241113</v>
@@ -27440,10 +27440,10 @@
         <v>300.1338842769231</v>
       </c>
       <c r="D47" t="n">
-        <v>22.02148609564698</v>
+        <v>22.02148609564697</v>
       </c>
       <c r="E47" t="n">
-        <v>13.62913851378318</v>
+        <v>13.62913851378319</v>
       </c>
     </row>
     <row r="48">
@@ -27459,7 +27459,7 @@
         <v>299.9727902294506</v>
       </c>
       <c r="D48" t="n">
-        <v>22.02148609564698</v>
+        <v>22.02148609564697</v>
       </c>
       <c r="E48" t="n">
         <v>13.62182320151167</v>
@@ -27478,7 +27478,7 @@
         <v>298.456295545055</v>
       </c>
       <c r="D49" t="n">
-        <v>22.02148609564698</v>
+        <v>22.02148609564697</v>
       </c>
       <c r="E49" t="n">
         <v>13.55295888064754</v>
@@ -27497,10 +27497,10 @@
         <v>334.8351848136264</v>
       </c>
       <c r="D50" t="n">
-        <v>27.7170694952267</v>
+        <v>27.71706949522669</v>
       </c>
       <c r="E50" t="n">
-        <v>12.08046849510155</v>
+        <v>12.08046849510156</v>
       </c>
     </row>
     <row r="51">
@@ -27516,10 +27516,10 @@
         <v>334.5702706153846</v>
       </c>
       <c r="D51" t="n">
-        <v>27.7170694952267</v>
+        <v>27.71706949522669</v>
       </c>
       <c r="E51" t="n">
-        <v>12.07091069541109</v>
+        <v>12.0709106954111</v>
       </c>
     </row>
     <row r="52">
@@ -27535,7 +27535,7 @@
         <v>332.1410708518681</v>
       </c>
       <c r="D52" t="n">
-        <v>27.7170694952267</v>
+        <v>27.71706949522669</v>
       </c>
       <c r="E52" t="n">
         <v>11.98326796088843</v>
@@ -27554,10 +27554,10 @@
         <v>336.8704927239561</v>
       </c>
       <c r="D53" t="n">
-        <v>28.51202684252052</v>
+        <v>28.51202684252051</v>
       </c>
       <c r="E53" t="n">
-        <v>11.81503141058968</v>
+        <v>11.81503141058969</v>
       </c>
     </row>
     <row r="54">
@@ -27573,10 +27573,10 @@
         <v>334.7220841648352</v>
       </c>
       <c r="D54" t="n">
-        <v>28.51202684252052</v>
+        <v>28.5120268425205</v>
       </c>
       <c r="E54" t="n">
-        <v>11.73968045181754</v>
+        <v>11.73968045181755</v>
       </c>
     </row>
     <row r="55">
@@ -27592,10 +27592,10 @@
         <v>331.9499550883516</v>
       </c>
       <c r="D55" t="n">
-        <v>28.51202684252052</v>
+        <v>28.51202684252051</v>
       </c>
       <c r="E55" t="n">
-        <v>11.64245379403573</v>
+        <v>11.64245379403574</v>
       </c>
     </row>
     <row r="56">
@@ -27611,7 +27611,7 @@
         <v>329.9367262325274</v>
       </c>
       <c r="D56" t="n">
-        <v>28.51202684252052</v>
+        <v>28.51202684252051</v>
       </c>
       <c r="E56" t="n">
         <v>11.57184398200996</v>
@@ -27630,7 +27630,7 @@
         <v>327.5751335485714</v>
       </c>
       <c r="D57" t="n">
-        <v>28.51202684252052</v>
+        <v>28.51202684252051</v>
       </c>
       <c r="E57" t="n">
         <v>11.48901603375501</v>
@@ -27649,7 +27649,7 @@
         <v>333.6696250747253</v>
       </c>
       <c r="D58" t="n">
-        <v>29.58282091361333</v>
+        <v>29.58282091361332</v>
       </c>
       <c r="E58" t="n">
         <v>11.27916861103595</v>
@@ -27668,7 +27668,7 @@
         <v>334.0981961208792</v>
       </c>
       <c r="D59" t="n">
-        <v>29.6588630924264</v>
+        <v>29.65886309242638</v>
       </c>
       <c r="E59" t="n">
         <v>11.26470003518758</v>
@@ -27687,10 +27687,10 @@
         <v>332.6221133657143</v>
       </c>
       <c r="D60" t="n">
-        <v>29.6588630924264</v>
+        <v>29.65886309242638</v>
       </c>
       <c r="E60" t="n">
-        <v>11.21493134545173</v>
+        <v>11.21493134545174</v>
       </c>
     </row>
     <row r="61">
@@ -27706,7 +27706,7 @@
         <v>331.4517690197802</v>
       </c>
       <c r="D61" t="n">
-        <v>29.6588630924264</v>
+        <v>29.65886309242638</v>
       </c>
       <c r="E61" t="n">
         <v>11.17547115635794</v>
@@ -27725,7 +27725,7 @@
         <v>338.4070822826374</v>
       </c>
       <c r="D62" t="n">
-        <v>30.91666952731508</v>
+        <v>30.91666952731506</v>
       </c>
       <c r="E62" t="n">
         <v>10.94578062438623</v>
@@ -27744,7 +27744,7 @@
         <v>337.7041371323077</v>
       </c>
       <c r="D63" t="n">
-        <v>30.91666952731508</v>
+        <v>30.91666952731506</v>
       </c>
       <c r="E63" t="n">
         <v>10.92304385612894</v>
@@ -27763,10 +27763,10 @@
         <v>339.2915739824176</v>
       </c>
       <c r="D64" t="n">
-        <v>31.20801100358216</v>
+        <v>31.20801100358215</v>
       </c>
       <c r="E64" t="n">
-        <v>10.87193842451134</v>
+        <v>10.87193842451135</v>
       </c>
     </row>
     <row r="65">
@@ -27782,7 +27782,7 @@
         <v>334.6419351652748</v>
       </c>
       <c r="D65" t="n">
-        <v>31.20801100358216</v>
+        <v>31.20801100358215</v>
       </c>
       <c r="E65" t="n">
         <v>10.72294979410458</v>
@@ -27801,10 +27801,10 @@
         <v>356.4361516892307</v>
       </c>
       <c r="D66" t="n">
-        <v>35.40534711718645</v>
+        <v>35.40534711718643</v>
       </c>
       <c r="E66" t="n">
-        <v>10.06729719410686</v>
+        <v>10.06729719410687</v>
       </c>
     </row>
     <row r="67">
@@ -27820,7 +27820,7 @@
         <v>349.9236171534065</v>
       </c>
       <c r="D67" t="n">
-        <v>34.12336679346627</v>
+        <v>34.12336679346624</v>
       </c>
       <c r="E67" t="n">
         <v>10.25466271459497</v>
@@ -27839,10 +27839,10 @@
         <v>344.5782724734066</v>
       </c>
       <c r="D68" t="n">
-        <v>33.08880958551386</v>
+        <v>33.08880958551384</v>
       </c>
       <c r="E68" t="n">
-        <v>10.41374037899089</v>
+        <v>10.4137403789909</v>
       </c>
     </row>
     <row r="69">
@@ -27858,10 +27858,10 @@
         <v>347.7716739019779</v>
       </c>
       <c r="D69" t="n">
-        <v>33.08880958551386</v>
+        <v>33.08880958551384</v>
       </c>
       <c r="E69" t="n">
-        <v>10.5102503915472</v>
+        <v>10.51025039154721</v>
       </c>
     </row>
     <row r="70">
@@ -27877,7 +27877,7 @@
         <v>351.1282640545055</v>
       </c>
       <c r="D70" t="n">
-        <v>33.08880958551386</v>
+        <v>33.08880958551384</v>
       </c>
       <c r="E70" t="n">
         <v>10.61169224438428</v>
@@ -27896,7 +27896,7 @@
         <v>351.6439501173626</v>
       </c>
       <c r="D71" t="n">
-        <v>33.08880958551385</v>
+        <v>33.08880958551383</v>
       </c>
       <c r="E71" t="n">
         <v>10.62727715267554</v>
@@ -27915,10 +27915,10 @@
         <v>345.3280371481318</v>
       </c>
       <c r="D72" t="n">
-        <v>31.91086108567557</v>
+        <v>31.91086108567555</v>
       </c>
       <c r="E72" t="n">
-        <v>10.82164584092485</v>
+        <v>10.82164584092486</v>
       </c>
     </row>
     <row r="73">
@@ -27934,7 +27934,7 @@
         <v>346.9452782861538</v>
       </c>
       <c r="D73" t="n">
-        <v>31.91086108567557</v>
+        <v>31.91086108567555</v>
       </c>
       <c r="E73" t="n">
         <v>10.87232580012997</v>
@@ -27953,10 +27953,10 @@
         <v>312.0884405947253</v>
       </c>
       <c r="D74" t="n">
-        <v>25.82093277484976</v>
+        <v>25.82093277484974</v>
       </c>
       <c r="E74" t="n">
-        <v>12.08664471249107</v>
+        <v>12.08664471249108</v>
       </c>
     </row>
     <row r="75">
@@ -27972,10 +27972,10 @@
         <v>312.3979251837362</v>
       </c>
       <c r="D75" t="n">
-        <v>25.82093277484976</v>
+        <v>25.82093277484975</v>
       </c>
       <c r="E75" t="n">
-        <v>12.09863051454205</v>
+        <v>12.09863051454206</v>
       </c>
     </row>
     <row r="76">
@@ -27991,10 +27991,10 @@
         <v>312.8709050347253</v>
       </c>
       <c r="D76" t="n">
-        <v>25.82093277484976</v>
+        <v>25.82093277484975</v>
       </c>
       <c r="E76" t="n">
-        <v>12.11694820488706</v>
+        <v>12.11694820488707</v>
       </c>
     </row>
     <row r="77">
@@ -28010,10 +28010,10 @@
         <v>310.1984566575824</v>
       </c>
       <c r="D77" t="n">
-        <v>25.381707532585</v>
+        <v>25.38170753258499</v>
       </c>
       <c r="E77" t="n">
-        <v>12.22133917741153</v>
+        <v>12.22133917741154</v>
       </c>
     </row>
     <row r="78">
@@ -28029,7 +28029,7 @@
         <v>254.8038257538461</v>
       </c>
       <c r="D78" t="n">
-        <v>15.31134777954465</v>
+        <v>15.31134777954466</v>
       </c>
       <c r="E78" t="n">
         <v>16.64150206908981</v>
@@ -28067,7 +28067,7 @@
         <v>249.6178962909889</v>
       </c>
       <c r="D80" t="n">
-        <v>14.85611458731971</v>
+        <v>14.8561145873197</v>
       </c>
       <c r="E80" t="n">
         <v>16.80236745777714</v>
@@ -28181,7 +28181,7 @@
         <v>136.3232243775824</v>
       </c>
       <c r="D86" t="n">
-        <v>7.745276202434011</v>
+        <v>7.74527620243401</v>
       </c>
       <c r="E86" t="n">
         <v>17.6008215607265</v>
@@ -28200,10 +28200,10 @@
         <v>137.369090523956</v>
       </c>
       <c r="D87" t="n">
-        <v>7.805118571946696</v>
+        <v>7.805118571946695</v>
       </c>
       <c r="E87" t="n">
-        <v>17.59987234757593</v>
+        <v>17.59987234757594</v>
       </c>
     </row>
     <row r="88">
@@ -28276,7 +28276,7 @@
         <v>92.91088673010984</v>
       </c>
       <c r="D91" t="n">
-        <v>5.271876022452656</v>
+        <v>5.271876022452657</v>
       </c>
       <c r="E91" t="n">
         <v>17.62387551118558</v>
@@ -28333,7 +28333,7 @@
         <v>59.16521491252744</v>
       </c>
       <c r="D94" t="n">
-        <v>3.355917954427953</v>
+        <v>3.355917954427954</v>
       </c>
       <c r="E94" t="n">
         <v>17.63011364281481</v>
@@ -28526,10 +28526,10 @@
         <v>76.0533070285714</v>
       </c>
       <c r="D6" t="n">
-        <v>1.579328664018362</v>
+        <v>1.579328664018361</v>
       </c>
       <c r="E6" t="n">
-        <v>48.15546552233486</v>
+        <v>48.15546552233487</v>
       </c>
     </row>
     <row r="7">
@@ -28716,7 +28716,7 @@
         <v>56.24774166461535</v>
       </c>
       <c r="D16" t="n">
-        <v>1.168664324538962</v>
+        <v>1.168664324538963</v>
       </c>
       <c r="E16" t="n">
         <v>48.12993815551361</v>
@@ -28757,7 +28757,7 @@
         <v>1.547122884465914</v>
       </c>
       <c r="E18" t="n">
-        <v>48.1558973327538</v>
+        <v>48.15589733275382</v>
       </c>
     </row>
     <row r="19">
@@ -30144,7 +30144,7 @@
         <v>5.356825851183538</v>
       </c>
       <c r="E91" t="n">
-        <v>46.30984062081256</v>
+        <v>46.30984062081255</v>
       </c>
     </row>
     <row r="92">
@@ -30429,10 +30429,10 @@
         <v>111.8985373635164</v>
       </c>
       <c r="D8" t="n">
-        <v>2.413964869530941</v>
+        <v>2.413964869530942</v>
       </c>
       <c r="E8" t="n">
-        <v>46.35466687021815</v>
+        <v>46.35466687021813</v>
       </c>
     </row>
     <row r="9">
@@ -34083,10 +34083,10 @@
         <v>47.96235398373623</v>
       </c>
       <c r="D4" t="n">
-        <v>1.813300766623508</v>
+        <v>1.813300766623509</v>
       </c>
       <c r="E4" t="n">
-        <v>26.45030260095542</v>
+        <v>26.45030260095541</v>
       </c>
     </row>
     <row r="5">
@@ -34102,10 +34102,10 @@
         <v>49.0857742496703</v>
       </c>
       <c r="D5" t="n">
-        <v>1.855778014887631</v>
+        <v>1.85577801488763</v>
       </c>
       <c r="E5" t="n">
-        <v>26.45024019892944</v>
+        <v>26.45024019892945</v>
       </c>
     </row>
     <row r="6">
@@ -34121,10 +34121,10 @@
         <v>26.035809272967</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9844417893733159</v>
+        <v>0.9844417893733156</v>
       </c>
       <c r="E6" t="n">
-        <v>26.44728165140276</v>
+        <v>26.44728165140277</v>
       </c>
     </row>
     <row r="7">
@@ -34143,7 +34143,7 @@
         <v>1.003047826500447</v>
       </c>
       <c r="E7" t="n">
-        <v>26.44749601637519</v>
+        <v>26.4474960163752</v>
       </c>
     </row>
     <row r="8">
@@ -34159,10 +34159,10 @@
         <v>26.05054804879119</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9849988328903777</v>
+        <v>0.984998832890378</v>
       </c>
       <c r="E8" t="n">
-        <v>26.44728823926475</v>
+        <v>26.44728823926474</v>
       </c>
     </row>
     <row r="9">
@@ -34181,7 +34181,7 @@
         <v>1.007988826776212</v>
       </c>
       <c r="E9" t="n">
-        <v>26.44755101758414</v>
+        <v>26.44755101758413</v>
       </c>
     </row>
     <row r="10">
@@ -34197,7 +34197,7 @@
         <v>19.80198908703294</v>
       </c>
       <c r="D10" t="n">
-        <v>0.7488484242097345</v>
+        <v>0.7488484242097346</v>
       </c>
       <c r="E10" t="n">
         <v>26.44325399753646</v>
@@ -34216,10 +34216,10 @@
         <v>19.18857086109887</v>
       </c>
       <c r="D11" t="n">
-        <v>0.7256666980073254</v>
+        <v>0.7256666980073259</v>
       </c>
       <c r="E11" t="n">
-        <v>26.44267804184831</v>
+        <v>26.44267804184829</v>
       </c>
     </row>
     <row r="12">
@@ -34254,10 +34254,10 @@
         <v>19.17943293890107</v>
       </c>
       <c r="D13" t="n">
-        <v>0.7253213675734077</v>
+        <v>0.725321367573408</v>
       </c>
       <c r="E13" t="n">
-        <v>26.44266913446469</v>
+        <v>26.44266913446468</v>
       </c>
     </row>
     <row r="14">
@@ -34273,7 +34273,7 @@
         <v>20.41177162945052</v>
       </c>
       <c r="D14" t="n">
-        <v>0.7718929327837257</v>
+        <v>0.7718929327837258</v>
       </c>
       <c r="E14" t="n">
         <v>26.4437861295585</v>
@@ -34292,10 +34292,10 @@
         <v>20.44435495780218</v>
       </c>
       <c r="D15" t="n">
-        <v>0.7731243059776214</v>
+        <v>0.7731243059776216</v>
       </c>
       <c r="E15" t="n">
-        <v>26.44381349768863</v>
+        <v>26.44381349768862</v>
       </c>
     </row>
     <row r="16">
@@ -34311,7 +34311,7 @@
         <v>20.99885491252744</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7940797762753408</v>
+        <v>0.7940797762753407</v>
       </c>
       <c r="E16" t="n">
         <v>26.44426358649167</v>
@@ -34330,7 +34330,7 @@
         <v>20.75522966109886</v>
       </c>
       <c r="D17" t="n">
-        <v>0.7848727565909073</v>
+        <v>0.7848727565909072</v>
       </c>
       <c r="E17" t="n">
         <v>26.44406941992629</v>
@@ -34482,10 +34482,10 @@
         <v>79.5457469907692</v>
       </c>
       <c r="D25" t="n">
-        <v>3.008059327670314</v>
+        <v>3.008059327670313</v>
       </c>
       <c r="E25" t="n">
-        <v>26.44420815076673</v>
+        <v>26.44420815076674</v>
       </c>
     </row>
     <row r="26">
@@ -34501,7 +34501,7 @@
         <v>173.6340593327472</v>
       </c>
       <c r="D26" t="n">
-        <v>6.589133893161904</v>
+        <v>6.589133893161903</v>
       </c>
       <c r="E26" t="n">
         <v>26.35157551024146</v>
@@ -34520,7 +34520,7 @@
         <v>175.4643669705494</v>
       </c>
       <c r="D27" t="n">
-        <v>6.65959490236021</v>
+        <v>6.659594902360209</v>
       </c>
       <c r="E27" t="n">
         <v>26.34760365204249</v>
@@ -34580,7 +34580,7 @@
         <v>10.8481217581227</v>
       </c>
       <c r="E30" t="n">
-        <v>25.58656248355387</v>
+        <v>25.58656248355386</v>
       </c>
     </row>
     <row r="31">
@@ -34653,10 +34653,10 @@
         <v>321.3750883872528</v>
       </c>
       <c r="D34" t="n">
-        <v>13.4111062691302</v>
+        <v>13.41110626913021</v>
       </c>
       <c r="E34" t="n">
-        <v>23.96335409905718</v>
+        <v>23.96335409905717</v>
       </c>
     </row>
     <row r="35">
@@ -34713,7 +34713,7 @@
         <v>13.56812816116157</v>
       </c>
       <c r="E37" t="n">
-        <v>23.82441830312901</v>
+        <v>23.82441830312902</v>
       </c>
     </row>
     <row r="38">
@@ -34767,10 +34767,10 @@
         <v>326.567124847912</v>
       </c>
       <c r="D40" t="n">
-        <v>13.86782067215197</v>
+        <v>13.86782067215198</v>
       </c>
       <c r="E40" t="n">
-        <v>23.54855406399167</v>
+        <v>23.54855406399166</v>
       </c>
     </row>
     <row r="41">
@@ -34805,7 +34805,7 @@
         <v>340.4169772404396</v>
       </c>
       <c r="D42" t="n">
-        <v>15.78672787313547</v>
+        <v>15.78672787313546</v>
       </c>
       <c r="E42" t="n">
         <v>21.56349181262146</v>
@@ -34824,10 +34824,10 @@
         <v>338.6988577661538</v>
       </c>
       <c r="D43" t="n">
-        <v>15.43539806662219</v>
+        <v>15.4353980666222</v>
       </c>
       <c r="E43" t="n">
-        <v>21.94299468690496</v>
+        <v>21.94299468690495</v>
       </c>
     </row>
     <row r="44">
@@ -34862,7 +34862,7 @@
         <v>337.1675648993407</v>
       </c>
       <c r="D45" t="n">
-        <v>15.16636669864806</v>
+        <v>15.16636669864807</v>
       </c>
       <c r="E45" t="n">
         <v>22.23126814739327</v>
@@ -34884,7 +34884,7 @@
         <v>17.3685352317065</v>
       </c>
       <c r="E46" t="n">
-        <v>20.77415732399204</v>
+        <v>20.77415732399203</v>
       </c>
     </row>
     <row r="47">
@@ -34903,7 +34903,7 @@
         <v>17.3685352317065</v>
       </c>
       <c r="E47" t="n">
-        <v>20.71593607324493</v>
+        <v>20.71593607324492</v>
       </c>
     </row>
     <row r="48">
@@ -34919,10 +34919,10 @@
         <v>362.996870912967</v>
       </c>
       <c r="D48" t="n">
-        <v>17.67801281765725</v>
+        <v>17.67801281765726</v>
       </c>
       <c r="E48" t="n">
-        <v>20.53380516561208</v>
+        <v>20.53380516561207</v>
       </c>
     </row>
     <row r="49">
@@ -34938,10 +34938,10 @@
         <v>361.9058664487912</v>
       </c>
       <c r="D49" t="n">
-        <v>17.67801281765725</v>
+        <v>17.67801281765726</v>
       </c>
       <c r="E49" t="n">
-        <v>20.47208983168687</v>
+        <v>20.47208983168686</v>
       </c>
     </row>
     <row r="50">
@@ -35014,7 +35014,7 @@
         <v>408.0451497059341</v>
       </c>
       <c r="D53" t="n">
-        <v>22.85322676346225</v>
+        <v>22.85322676346226</v>
       </c>
       <c r="E53" t="n">
         <v>17.85503438658023</v>
@@ -35033,7 +35033,7 @@
         <v>411.5172417217582</v>
       </c>
       <c r="D54" t="n">
-        <v>23.24380166892377</v>
+        <v>23.24380166892378</v>
       </c>
       <c r="E54" t="n">
         <v>17.70438620941873</v>
@@ -35052,7 +35052,7 @@
         <v>406.9943967731868</v>
       </c>
       <c r="D55" t="n">
-        <v>23.24380166892377</v>
+        <v>23.24380166892378</v>
       </c>
       <c r="E55" t="n">
         <v>17.50980336909884</v>
@@ -35074,7 +35074,7 @@
         <v>23.49272339666867</v>
       </c>
       <c r="E56" t="n">
-        <v>17.41679206665082</v>
+        <v>17.41679206665081</v>
       </c>
     </row>
     <row r="57">
@@ -35109,7 +35109,7 @@
         <v>419.6166915178022</v>
       </c>
       <c r="D58" t="n">
-        <v>24.805052361948</v>
+        <v>24.80505236194801</v>
       </c>
       <c r="E58" t="n">
         <v>16.91658156551654</v>
@@ -35147,7 +35147,7 @@
         <v>421.9856090347253</v>
       </c>
       <c r="D60" t="n">
-        <v>25.42728259270169</v>
+        <v>25.4272825927017</v>
       </c>
       <c r="E60" t="n">
         <v>16.59578083093497</v>
@@ -35166,10 +35166,10 @@
         <v>418.8414437907692</v>
       </c>
       <c r="D61" t="n">
-        <v>25.42728259270169</v>
+        <v>25.4272825927017</v>
       </c>
       <c r="E61" t="n">
-        <v>16.47212761583056</v>
+        <v>16.47212761583055</v>
       </c>
     </row>
     <row r="62">
@@ -35185,10 +35185,10 @@
         <v>429.0346540206593</v>
       </c>
       <c r="D62" t="n">
-        <v>26.67997379553694</v>
+        <v>26.67997379553695</v>
       </c>
       <c r="E62" t="n">
-        <v>16.08077494035728</v>
+        <v>16.08077494035727</v>
       </c>
     </row>
     <row r="63">
@@ -35204,7 +35204,7 @@
         <v>432.2321402465934</v>
       </c>
       <c r="D63" t="n">
-        <v>27.0791338190925</v>
+        <v>27.07913381909251</v>
       </c>
       <c r="E63" t="n">
         <v>15.96181558591222</v>
@@ -35223,10 +35223,10 @@
         <v>435.0898017481318</v>
       </c>
       <c r="D64" t="n">
-        <v>27.43837967857641</v>
+        <v>27.43837967857642</v>
       </c>
       <c r="E64" t="n">
-        <v>15.85697868623945</v>
+        <v>15.85697868623944</v>
       </c>
     </row>
     <row r="65">
@@ -35242,10 +35242,10 @@
         <v>428.9552856237361</v>
       </c>
       <c r="D65" t="n">
-        <v>27.43837967857641</v>
+        <v>27.43837967857642</v>
       </c>
       <c r="E65" t="n">
-        <v>15.63340440101351</v>
+        <v>15.6334044010135</v>
       </c>
     </row>
     <row r="66">
@@ -35261,7 +35261,7 @@
         <v>455.0936698852747</v>
       </c>
       <c r="D66" t="n">
-        <v>30.88417492678299</v>
+        <v>30.884174926783</v>
       </c>
       <c r="E66" t="n">
         <v>14.73549709403485</v>
@@ -35280,10 +35280,10 @@
         <v>450.9030872017581</v>
       </c>
       <c r="D67" t="n">
-        <v>30.31801976484889</v>
+        <v>30.3180197648489</v>
       </c>
       <c r="E67" t="n">
-        <v>14.87244518933064</v>
+        <v>14.87244518933063</v>
       </c>
     </row>
     <row r="68">
@@ -35299,7 +35299,7 @@
         <v>449.4377677331868</v>
       </c>
       <c r="D68" t="n">
-        <v>30.12128836075368</v>
+        <v>30.1212883607537</v>
       </c>
       <c r="E68" t="n">
         <v>14.92093440195534</v>
@@ -35318,7 +35318,7 @@
         <v>441.6806175402197</v>
       </c>
       <c r="D69" t="n">
-        <v>29.09049403691128</v>
+        <v>29.09049403691129</v>
       </c>
       <c r="E69" t="n">
         <v>15.18298785093839</v>
@@ -35337,7 +35337,7 @@
         <v>453.2321048742857</v>
       </c>
       <c r="D70" t="n">
-        <v>29.09049403691128</v>
+        <v>29.09049403691129</v>
       </c>
       <c r="E70" t="n">
         <v>15.58007589349308</v>
@@ -35356,7 +35356,7 @@
         <v>445.9307434523077</v>
       </c>
       <c r="D71" t="n">
-        <v>28.16077447984162</v>
+        <v>28.16077447984163</v>
       </c>
       <c r="E71" t="n">
         <v>15.83517327520658</v>
@@ -35375,10 +35375,10 @@
         <v>450.2238132026373</v>
       </c>
       <c r="D72" t="n">
-        <v>28.16077447984163</v>
+        <v>28.16077447984164</v>
       </c>
       <c r="E72" t="n">
-        <v>15.98762184345895</v>
+        <v>15.98762184345894</v>
       </c>
     </row>
     <row r="73">
@@ -35394,10 +35394,10 @@
         <v>445.5410777841757</v>
       </c>
       <c r="D73" t="n">
-        <v>27.57802576094459</v>
+        <v>27.57802576094461</v>
       </c>
       <c r="E73" t="n">
-        <v>16.15565529042117</v>
+        <v>16.15565529042116</v>
       </c>
     </row>
     <row r="74">
@@ -35413,7 +35413,7 @@
         <v>405.0836300334066</v>
       </c>
       <c r="D74" t="n">
-        <v>22.79696628790177</v>
+        <v>22.79696628790179</v>
       </c>
       <c r="E74" t="n">
         <v>17.76919020353959</v>
@@ -35451,7 +35451,7 @@
         <v>399.7657383283516</v>
       </c>
       <c r="D76" t="n">
-        <v>22.20234320079684</v>
+        <v>22.20234320079685</v>
       </c>
       <c r="E76" t="n">
         <v>18.00556521052264</v>
@@ -35470,10 +35470,10 @@
         <v>394.6167538259339</v>
       </c>
       <c r="D77" t="n">
-        <v>21.63409388778032</v>
+        <v>21.63409388778033</v>
       </c>
       <c r="E77" t="n">
-        <v>18.24050297058325</v>
+        <v>18.24050297058324</v>
       </c>
     </row>
     <row r="78">
@@ -35508,10 +35508,10 @@
         <v>324.0348582092308</v>
       </c>
       <c r="D79" t="n">
-        <v>13.63606214978826</v>
+        <v>13.63606214978827</v>
       </c>
       <c r="E79" t="n">
-        <v>23.76308164701804</v>
+        <v>23.76308164701803</v>
       </c>
     </row>
     <row r="80">
@@ -35584,7 +35584,7 @@
         <v>252.507511410989</v>
       </c>
       <c r="D83" t="n">
-        <v>9.733209220323916</v>
+        <v>9.733209220323918</v>
       </c>
       <c r="E83" t="n">
         <v>25.94288334866243</v>
@@ -35641,7 +35641,7 @@
         <v>191.3136029182417</v>
       </c>
       <c r="D86" t="n">
-        <v>7.272450791640984</v>
+        <v>7.272450791640983</v>
       </c>
       <c r="E86" t="n">
         <v>26.3066204776716</v>
@@ -35679,7 +35679,7 @@
         <v>193.1329048905494</v>
       </c>
       <c r="D88" t="n">
-        <v>7.343162400456031</v>
+        <v>7.343162400456033</v>
       </c>
       <c r="E88" t="n">
         <v>26.30105319181764</v>
@@ -35698,7 +35698,7 @@
         <v>189.6053556316484</v>
       </c>
       <c r="D89" t="n">
-        <v>7.2061314812625</v>
+        <v>7.206131481262501</v>
       </c>
       <c r="E89" t="n">
         <v>26.311670294202</v>
@@ -35736,7 +35736,7 @@
         <v>129.6172607854945</v>
       </c>
       <c r="D91" t="n">
-        <v>4.906957553158348</v>
+        <v>4.906957553158349</v>
       </c>
       <c r="E91" t="n">
         <v>26.41499531661258</v>
@@ -35796,7 +35796,7 @@
         <v>3.229121460199138</v>
       </c>
       <c r="E94" t="n">
-        <v>26.44217382714826</v>
+        <v>26.44217382714825</v>
       </c>
     </row>
     <row r="95">
@@ -35831,10 +35831,10 @@
         <v>86.60890223076919</v>
       </c>
       <c r="D96" t="n">
-        <v>3.275465241517671</v>
+        <v>3.275465241517672</v>
       </c>
       <c r="E96" t="n">
-        <v>26.44171006090096</v>
+        <v>26.44171006090095</v>
       </c>
     </row>
     <row r="97">

</xml_diff>